<commit_message>
Reglas v3 (22-10-2026): hoja Novedades para avisar a los responsables qué cambió
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -8,26 +8,27 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subitems" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respaldos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TiposActividad" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificadores" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoFinanciables" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasGenerales" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plazos" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Novedades" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subitems" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Respaldos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TiposActividad" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificadores" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoFinanciables" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasGenerales" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plazos" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Subitems'!$A$1:$F$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Respaldos'!$A$1:$I$83</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TiposActividad'!$A$1:$D$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Verificadores'!$A$1:$G$183</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'NoFinanciables'!$A$1:$H$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ReglasGenerales'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Plazos'!$A$1:$J$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Subitems'!$A$1:$F$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Respaldos'!$A$1:$I$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TiposActividad'!$A$1:$D$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Verificadores'!$A$1:$G$183</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'NoFinanciables'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ReglasGenerales'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Plazos'!$A$1:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -469,7 +470,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2">
@@ -580,27 +581,47 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>9. Novedades: si la versión nueva cambia algo para los responsables, agrega en la hoja Novedades una fila por cambio, con el número de la versión nueva. El programa las muestra hasta que el responsable las marca como leídas.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Pendiente de validar</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -612,6 +633,264 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>ComoEvitarlo</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Falta documentación de respaldo</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Usa el checklist de cada gasto y no entregues hasta tener todos los documentos.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Sección 2.03; Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Documentos que no son originales</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Guarda los originales o los archivos electrónicos que te entregó el proveedor.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Gastos sin el detalle de lo comprado</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Pide boletas o facturas que detallen qué compraste.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Gastos rendidos en el ítem equivocado</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Rinde cada gasto en el ítem y subítem de tu presupuesto aprobado.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Faltan firmas</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Revisa que contratos, recepciones conformes, listas y declaraciones estén firmados.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Entrega fuera de plazo</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Anota las fechas del calendario de esta guía y pide la prórroga a tiempo.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Documentos de otro período</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Revisa que la fecha de cada documento esté dentro del período del convenio.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Documentación improcedente o adulterada</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Nunca corrijas a mano una boleta: pide una nueva al proveedor.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>No cumplir el calendario de actividades</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Si una fecha cambia, pide la modificación antes.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Faltan medios de verificación</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Junta al menos 3 verificadores por actividad mientras la haces, no al final.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Piezas gráficas sin logo o sin mención del financiamiento</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Incluye el logo y la mención autorizados por el Ministerio en toda pieza de difusión.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Fotografías sin fecha</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Activa la fecha en tu cámara o celular, o anótala en cada foto.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Listas de participantes sin fecha</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Pon fecha, nombre de la actividad y firmas en cada lista.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5759,6 +6038,228 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Novedad</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Todos los beneficiarios rinden en SISREC, sin importar el monto del proyecto.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/566, punto V</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Si tu convenio se rige por la Res. 2/2026, para recibir recursos de un nuevo convenio basta con haber presentado tus rendiciones anteriores: no tienen que estar aprobadas.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 38; Memo 02/566, punto IV</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Si tu garantía es una letra de cambio, renuévala cada 6 meses desde su emisión.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1264</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Plazos para responder observaciones con la Res. 2/2026: hasta el 31-12-2026 siguen los del instructivo (10 días hábiles lo financiero y 20 las actividades); después, 40 días hábiles en 2027, 30 en 2028 y 20 desde 2029.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>En alimentación y alojamiento, pide factura a tu nombre con la fecha, el número de personas y el detalle. En traslados, lleva una planilla firmada con cada persona, tramo y monto.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3391, Anexo A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo tipo de gasto: viáticos. Si pagas viático a alguien, no rindas aparte su alojamiento, alimentación ni movilización en la ciudad.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3391, Anexo A letra d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Finiquitos e indemnizaciones: consulta a tu supervisor antes de pagarlos con los fondos, porque las normas no coinciden.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096; Rex 3391, Anexo A letra j)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Los recursos de los convenios con presupuesto 2026 se transfieren en una sola cuota.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/064; Dictamen CGR OF192150</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Fondo Audiovisual: si tu línea tiene obligación de reembolso, la guía explica cuándo devolver y qué informar cada año.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3390</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Bases 2027 de Fondart Regional y Libro: sus reglas aparecen en la guía si tu convenio se firma desde el 01-01-2027.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Bases de la Convocatoria 2027, tanda 1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6678,7 +7179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10066,7 +10567,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10665,7 +11166,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16004,7 +16505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17045,7 +17546,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18547,7 +19048,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19482,262 +19983,4 @@
   <autoFilter ref="A1:J15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>ComoEvitarlo</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Falta documentación de respaldo</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Usa el checklist de cada gasto y no entregues hasta tener todos los documentos.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.1, Sección 2.03; Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Documentos que no son originales</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Guarda los originales o los archivos electrónicos que te entregó el proveedor.</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Gastos sin el detalle de lo comprado</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Pide boletas o facturas que detallen qué compraste.</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Gastos rendidos en el ítem equivocado</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Rinde cada gasto en el ítem y subítem de tu presupuesto aprobado.</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Faltan firmas</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Revisa que contratos, recepciones conformes, listas y declaraciones estén firmados.</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Entrega fuera de plazo</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Anota las fechas del calendario de esta guía y pide la prórroga a tiempo.</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Documentos de otro período</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Revisa que la fecha de cada documento esté dentro del período del convenio.</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Documentación improcedente o adulterada</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Nunca corrijas a mano una boleta: pide una nueva al proveedor.</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 4.06</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>No cumplir el calendario de actividades</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Si una fecha cambia, pide la modificación antes.</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Faltan medios de verificación</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Junta al menos 3 verificadores por actividad mientras la haces, no al final.</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°3</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Piezas gráficas sin logo o sin mención del financiamiento</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Incluye el logo y la mención autorizados por el Ministerio en toda pieza de difusión.</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°4</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Fotografías sin fecha</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Activa la fecha en tu cámara o celular, o anótala en cada foto.</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°5</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Listas de participantes sin fecha</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Pon fecha, nombre de la actividad y firmas en cada lista.</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.1, Sección 2.03 N°6</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:C14"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Reglas v4 (22-10-2026): documentos de Biblioteca Transferencias (SISREC según la norma, cambios dentro de un ítem, fuerza mayor y otros)
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2">
@@ -491,7 +491,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Reglas v2. Capa común: Rex 3092 a 3097, 3390 y 3391 de 2025 y Rex 1523 de 2024 (Subsecretaría de las Culturas y las Artes); Memos 02/1264, 02/566, 02/580 y 02/064; Res. 30/2015 y Res. 2/2026 de Contraloría. Capa por fondo: bases de la Convocatoria 2027, tanda 1 (Fondart Regional y Libro), para convenios firmados desde el 01-01-2027.</t>
+          <t>Reglas v2. Capa común: Rex 3092 a 3097, 3390 y 3391 de 2025 y Rex 1523 de 2024 (Subsecretaría de las Culturas y las Artes); Memos 02/1264, 02/566, 02/580, 02/064, 02/872, 02/978, 02/1283, 02/490, 02/306, 06/455 y 06/561; dictámenes de la CGR; Res. 30/2015 y Res. 2/2026 de Contraloría. Capa por fondo: bases de la Convocatoria 2027, tanda 1 (Fondart Regional y Libro), para convenios firmados desde el 01-01-2027.</t>
         </is>
       </c>
     </row>
@@ -606,22 +606,34 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 4</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -4364,7 +4376,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Las bases 2027 lo permiten; el instructivo de rendición (Rex 3096) pide autorización con 15 días hábiles de anticipación. Pendiente de confirmar con Jurídico.</t>
+          <t>Jurídico aplicó esta misma cláusula en 2026 (Memo 06/455): mover dinero dentro de un ítem no requiere autorización si el total del ítem no sube.</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -4399,7 +4411,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Las bases 2027 lo permiten; el instructivo de rendición (Rex 3096) pide autorización con 15 días hábiles de anticipación. Pendiente de confirmar con Jurídico.</t>
+          <t>Jurídico aplicó esta misma cláusula en 2026 (Memo 06/455): mover dinero dentro de un ítem no requiere autorización si el total del ítem no sube.</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -4434,7 +4446,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Las bases 2027 lo permiten; el instructivo de rendición (Rex 3096) pide autorización con 15 días hábiles de anticipación. Pendiente de confirmar con Jurídico.</t>
+          <t>Jurídico aplicó esta misma cláusula en 2026 (Memo 06/455): mover dinero dentro de un ítem no requiere autorización si el total del ítem no sube.</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -4469,7 +4481,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Las bases 2027 lo permiten; el instructivo de rendición (Rex 3096) pide autorización con 15 días hábiles de anticipación. Pendiente de confirmar con Jurídico.</t>
+          <t>Jurídico aplicó esta misma cláusula en 2026 (Memo 06/455): mover dinero dentro de un ítem no requiere autorización si el total del ítem no sube.</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -4504,7 +4516,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Las bases 2027 lo permiten; el instructivo de rendición (Rex 3096) pide autorización con 15 días hábiles de anticipación. Pendiente de confirmar con Jurídico.</t>
+          <t>Jurídico aplicó esta misma cláusula en 2026 (Memo 06/455): mover dinero dentro de un ítem no requiere autorización si el total del ítem no sube.</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -4539,7 +4551,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Las bases 2027 lo permiten; el instructivo de rendición (Rex 3096) pide autorización con 15 días hábiles de anticipación. Pendiente de confirmar con Jurídico.</t>
+          <t>Jurídico aplicó esta misma cláusula en 2026 (Memo 06/455): mover dinero dentro de un ítem no requiere autorización si el total del ítem no sube.</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -4574,7 +4586,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Las bases 2027 lo permiten; el instructivo de rendición (Rex 3096) pide autorización con 15 días hábiles de anticipación. Pendiente de confirmar con Jurídico.</t>
+          <t>Jurídico aplicó esta misma cláusula en 2026 (Memo 06/455): mover dinero dentro de un ítem no requiere autorización si el total del ítem no sube.</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -6038,7 +6050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6078,7 +6090,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Todos los beneficiarios rinden en SISREC, sin importar el monto del proyecto.</t>
+          <t>Si tu convenio se firmó desde el 01-07-2026, rindes en SISREC sin importar el monto del proyecto.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -6246,6 +6258,114 @@
       <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Bases de la Convocatoria 2027, tanda 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Corrección: si tu convenio se firmó hasta el 30-06-2026 y es de menos de 500 UTM, revisa si te exceptúa de SISREC; en ese caso rindes en papel.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/872</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Para recibir recursos de un nuevo convenio basta con haber presentado tus rendiciones anteriores, con cualquiera de las dos normas; tener gastos rechazados no lo impide.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/978</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Cambios al proyecto: mover dinero entre ítems siempre requiere autorización y anexo; dentro de un mismo ítem, revisa la cláusula de modificaciones de tu convenio.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Memo 06/455</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Gastos anteriores al convenio: solo valen si tu convenio y la resolución que lo aprueba lo autorizan expresamente.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Memo 06/561</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en la guía: qué hacer ante fuerza mayor o catástrofe, pagos con tarjeta de crédito, documentos perdidos y copias de facturas.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1283; Dictámenes CGR 16.096, 19.889 y 85.710</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>46317</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Inicio de actividades en el SII: si tu actividad no produce renta, puedes eximirte con una declaración jurada.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/490</t>
         </is>
       </c>
     </row>
@@ -8562,7 +8682,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.2, Art. IV; Rex 3391, Anexo A letra c)</t>
+          <t>Rex 3096, Instr. 4.2, Art. IV; Rex 3391, Anexo A letra c); Memo 02/306 (28-03-2019)</t>
         </is>
       </c>
       <c r="F37" s="5" t="n"/>
@@ -8675,7 +8795,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.2, Art. IV; Rex 3391, Anexo A letra c)</t>
+          <t>Rex 3096, Instr. 4.2, Art. IV; Rex 3391, Anexo A letra c); Memo 02/306 (28-03-2019)</t>
         </is>
       </c>
       <c r="F40" s="5" t="n"/>
@@ -17552,7 +17672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -17743,7 +17863,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Presenta documentos originales, sin alteraciones ni enmiendas: un documento corregido a mano o adulterado se rechaza.</t>
+          <t>Presenta documentos originales, sin alteraciones ni enmiendas: un documento corregido a mano o adulterado se rechaza. Una copia de la factura (como la «tercera copia») no acredita el gasto.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -17753,7 +17873,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.2, Art. II</t>
+          <t>Rex 3096, Instr. 4.2, Art. II; Dictamen CGR N° 85.710 de 2015</t>
         </is>
       </c>
       <c r="F5" s="5" t="n"/>
@@ -17823,7 +17943,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Solo valen gastos hechos después de la total tramitación de la resolución que aprueba tu convenio y antes de la entrega del informe final (o de la prórroga). Un gasto anterior vale solo si tu convenio lo autoriza expresamente.</t>
+          <t>Solo valen gastos hechos después de la total tramitación de la resolución que aprueba tu convenio y antes de la entrega del informe final (o de la prórroga). Un gasto anterior vale solo si tu convenio y la resolución que lo aprueba lo autorizan expresamente, con sus razones: no basta la resolución que te seleccionó.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -17833,7 +17953,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.2, Art. II; Res. 30/2015 CGR, art. 13</t>
+          <t>Rex 3096, Instr. 4.2, Art. II; Res. 30/2015 CGR, art. 13; Memo 06/561 (13-05-2026)</t>
         </is>
       </c>
       <c r="F7" s="5" t="n"/>
@@ -17864,7 +17984,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Solo valen gastos hechos después de la total tramitación de la resolución que aprueba tu convenio y antes de la entrega del informe final (o de la prórroga). Un gasto anterior vale solo si tu convenio lo autoriza expresamente.</t>
+          <t>Solo valen gastos hechos después de la total tramitación de la resolución que aprueba tu convenio y antes de la entrega del informe final (o de la prórroga). Un gasto anterior vale solo si tu convenio y la resolución que lo aprueba lo autorizan expresamente, con sus razones: no basta la resolución que te seleccionó.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -17874,7 +17994,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.2, Art. II; Res. 2/2026 CGR, art. 36</t>
+          <t>Rex 3096, Instr. 4.2, Art. II; Res. 2/2026 CGR, art. 36; Memo 06/561 (13-05-2026)</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
@@ -18100,7 +18220,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>No hagas cambios (fechas, lugares, equipo, presupuesto) sin pedir autorización antes.</t>
+          <t>Mover dinero entre ítems (por ejemplo, de Operación a Personal) siempre requiere autorización previa y un anexo del convenio. Dentro de un mismo ítem, muchos convenios lo permiten sin autorización, salvo en alojamiento, alimentación y traslado: revisa la cláusula de modificaciones de tu convenio y, si dudas, pide autorización. Para cambiar fechas, lugares o el equipo, pide autorización antes.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -18110,7 +18230,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Rex 3094, Art. V N°1; Rex 3096, Instr. 4.3, Sección 3.01</t>
+          <t>Rex 3094, Art. V N°1; Rex 3096, Instr. 4.3, Sección 3.01; Memo 06/455 (21-04-2026)</t>
         </is>
       </c>
       <c r="F14" s="5" t="n"/>
@@ -18424,10 +18544,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Rex 3391, punto 5.3.1; Res. 2/2026 CGR, art. 27; Memo 02/566, punto V</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="n"/>
+          <t>Res. 2/2026 CGR, art. 27; Memo 02/566, punto V</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>46204</v>
+      </c>
       <c r="G22" s="5" t="n"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -18443,17 +18565,17 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Proyecto</t>
+          <t>Entrega</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Rendiciones pendientes</t>
+          <t>Sistema de rendición</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Mientras tengas rendiciones pendientes de otros proyectos con el Ministerio, no podrás firmar nuevos convenios.</t>
+          <t>Desde octubre de 2023 se rinde en SISREC, el sistema de rendición de Contraloría. Si tu convenio es de menos de 500 UTM, revisa si trae la cláusula que te exceptúa: en ese caso rindes en papel, con los formatos de tu convenio.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -18463,7 +18585,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Rex 3094 (certificado de habilitación); Rex 3096, Instr. 4.1 (certificado de rechazo); Res. 30/2015 CGR, art. 18</t>
+          <t>Rex 1858/2023 CGR, art. 4; Memo 02/872 (07-11-2023)</t>
         </is>
       </c>
       <c r="F23" s="5" t="n"/>
@@ -18494,7 +18616,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Para recibir recursos de un nuevo convenio, debes haber presentado las rendiciones que te correspondían en otros proyectos con el Ministerio. Basta con presentarlas: no es necesario que ya estén aprobadas.</t>
+          <t>Para recibir recursos de un nuevo convenio, debes haber presentado las rendiciones que te correspondían en otros proyectos con el Ministerio. Basta con presentarlas: no necesitan estar aprobadas, y tener gastos rechazados no lo impide.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -18504,12 +18626,10 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Res. 2/2026 CGR, art. 38; Memo 02/566, punto IV</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>46204</v>
-      </c>
+          <t>Res. 30/2015 CGR, art. 18; Res. 2/2026 CGR, art. 38; Memo 02/978 (nov-2023); Memo 02/566, punto IV</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -18654,7 +18774,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Cuando el Ministerio cargue la transferencia en SISREC, acéptala y carga tu comprobante de ingreso. Desde el mes siguiente rindes cada mes, dentro de los primeros 15 días hábiles, salvo que tu convenio fije otra periodicidad.</t>
+          <t>Si rindes en SISREC: cuando el Ministerio cargue la transferencia en SISREC, acéptala y carga tu comprobante de ingreso. Desde el mes siguiente rindes cada mes, dentro de los primeros 15 días hábiles, salvo que tu convenio fije otra periodicidad.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -18693,7 +18813,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Si en un mes no tuviste gastos, o tu convenio no te pide rendir ese mes, ingresa en SISREC una rendición «sin movimiento».</t>
+          <t>Si rindes en SISREC: si en un mes no tuviste gastos, o tu convenio no te pide rendir ese mes, ingresa en SISREC una rendición «sin movimiento».</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -18812,7 +18932,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Las normas no coinciden: el instructivo de rendición los declara no financiables; el procedimiento de revisión en SISREC acepta las indemnizaciones obligatorias por ley que se generen durante el convenio y se relacionen con el proyecto. Consulta a tu supervisor antes de pagarlos con los fondos.</t>
+          <t>Las normas no coinciden: el instructivo de rendición los declara no financiables; el procedimiento de revisión en SISREC acepta las indemnizaciones obligatorias por ley que se generen durante el convenio y se relacionen con el proyecto. Consulta a tu supervisor antes de pagarlos con los fondos. Las indemnizaciones voluntarias (por ejemplo, por mutuo acuerdo) nunca se pueden pagar con los fondos.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -18822,7 +18942,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.2, Sección 2.01 N°2; Rex 3391, Anexo A letra j)</t>
+          <t>Rex 3096, Instr. 4.2, Sección 2.01 N°2; Rex 3391, Anexo A letra j); Dictamen CGR N° 9.569 de 2019</t>
         </is>
       </c>
       <c r="F32" s="5" t="n"/>
@@ -19032,6 +19152,201 @@
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Gastos</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Honorarios o contrato de trabajo</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Si postulaste a alguien con boleta de honorarios y en realidad cumple horario o trabaja de forma continua, puedes pagarle con contrato de trabajo dentro del ítem Personal, si tu convenio permite mover dinero dentro del ítem y el total del ítem no sube: los mayores costos (por ejemplo, las cotizaciones) los cubres tú. Avísale a tu supervisor antes.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Memo 06/455 (21-04-2026)</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Gastos</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Pagos con tarjeta de crédito</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Paga con débito, transferencia o efectivo. La tarjeta de crédito se acepta solo en casos excepcionales (por ejemplo, para no llevar efectivo en el extranjero); entonces rinde el voucher, la boleta o factura y el estado de cuenta pagado. Los intereses de pagar en cuotas no se financian.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen CGR N° 16.096 de 2017</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Gastos</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Si pierdes un documento</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Avisa de inmediato a tu supervisor y pide un duplicado al proveedor. Solo en casos especiales, que decide el Ministerio, se acepta otra prueba en vez del documento original.</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Dictámenes CGR N° 19.889 de 2012 y 90.073 de 2016</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Fuerza mayor o catástrofe</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Si un hecho que no podías prever ni evitar (un temporal, un incendio, una catástrofe declarada en tu región) te impide ejecutar, avisa a tu supervisor y acredítalo con documentos: el Ministerio lo evalúa caso a caso. Si la actividad se suspende, se hace en una nueva fecha con una prórroga y los mayores costos son tuyos; si se cancela, se pone término al convenio: rindes lo ya gastado y devuelves lo que no alcanzaste a usar. En julio de 2026, por ejemplo, La Araucanía y otras regiones fueron declaradas zona afectada por catástrofe.</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1283 (25-11-2019); Memo 02/139 (10-02-2023); Decreto N° 113 de 2026 (Interior)</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Inicio de actividades</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Para firmar el convenio pueden pedirte acreditar tu inicio de actividades en el SII. Si tu actividad no produce renta, puedes eximirte con una declaración jurada (formato del Memo 02/490); lo que declares es tu responsabilidad.</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/490 (20-05-2026); Oficio SII N° 88 (07-05-2026); Código Tributario, art. 68</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>Todas</t>
         </is>
@@ -19184,7 +19499,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pide cualquier cambio (fechas, equipo, presupuesto) con 15 días hábiles de anticipación y espera la autorización antes de hacerlo.</t>
+          <t>Pide los cambios que necesitan autorización (fechas, equipo, mover dinero entre ítems) con 15 días hábiles de anticipación y espera la autorización antes de hacerlos.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Reglas v5 (22-10-2026): filas Programa y Descarga para el aviso de versión nueva del programa
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -77,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -91,6 +91,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -470,7 +473,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
@@ -484,156 +487,195 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Contenido</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Reglas v2. Capa común: Rex 3092 a 3097, 3390 y 3391 de 2025 y Rex 1523 de 2024 (Subsecretaría de las Culturas y las Artes); Memos 02/1264, 02/566, 02/580, 02/064, 02/872, 02/978, 02/1283, 02/490, 02/306, 06/455 y 06/561; dictámenes de la CGR; Res. 30/2015 y Res. 2/2026 de Contraloría. Capa por fondo: bases de la Convocatoria 2027, tanda 1 (Fondart Regional y Libro), para convenios firmados desde el 01-01-2027.</t>
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>0.2.0-prueba</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="2" t="inlineStr"/>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Descarga</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Contenido</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Reglas v2. Capa común: Rex 3092 a 3097, 3390 y 3391 de 2025 y Rex 1523 de 2024 (Subsecretaría de las Culturas y las Artes); Memos 02/1264, 02/566, 02/580, 02/064, 02/872, 02/978, 02/1283, 02/490, 02/306, 06/455 y 06/561; dictámenes de la CGR; Res. 30/2015 y Res. 2/2026 de Contraloría. Capa por fondo: bases de la Convocatoria 2027, tanda 1 (Fondart Regional y Libro), para convenios firmados desde el 01-01-2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Cómo editar</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>1. No cambies los nombres de las hojas ni de las columnas (fila 1): el programa los busca tal cual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>2. Una regla por fila.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>3. VigenteDesde y VigenteHasta: rango de fechas de la resolución que aprueba el convenio en que aplica la regla. Vacío = sin límite.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>4. Fondo y Linea: "Todos" y "Todas" para reglas comunes. Para un fondo o una línea, escribe su nombre o una parte, como aparece en la postulación (ej. Fondart Regional / Creación Artística): el programa busca esas palabras completas dentro del nombre.</t>
+          <t>2. Una regla por fila.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>5. TipoPersona: Todas, Natural o Juridica.</t>
+          <t>3. VigenteDesde y VigenteHasta: rango de fechas de la resolución que aprueba el convenio en que aplica la regla. Vacío = sin límite.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>6. PalabrasClave: en minúsculas y separadas por punto y coma; las tildes no importan.</t>
+          <t>4. Fondo y Linea: "Todos" y "Todas" para reglas comunes. Para un fondo o una línea, escribe su nombre o una parte, como aparece en la postulación (ej. Fondart Regional / Creación Artística): el programa busca esas palabras completas dentro del nombre.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>7. Plazos: no cambies la columna Clave, la usa el programa. Puedes cambiar Cantidad, Unidad y los textos.</t>
+          <t>5. TipoPersona: Todas, Natural o Juridica.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>6b. Las palabras clave se comparan por palabra completa (también en plural). Si un gasto calza con varios subítems, gana el de mayor Prioridad; a igual prioridad, el de la palabra clave más larga.</t>
+          <t>6. PalabrasClave: en minúsculas y separadas por punto y coma; las tildes no importan.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>6c. ReglasGenerales.Seccion: Gastos, Proyecto, Entrega o Cofinanciamiento. Define en qué parte de la guía aparece la regla.</t>
+          <t>7. Plazos: no cambies la columna Clave, la usa el programa. Puedes cambiar Cantidad, Unidad y los textos.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>6d. En los textos puedes escribir [tu folio]: el programa lo reemplaza por el folio del proyecto.</t>
+          <t>6b. Las palabras clave se comparan por palabra completa (también en plural). Si un gasto calza con varios subítems, gana el de mayor Prioridad; a igual prioridad, el de la palabra clave más larga.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>8. Al publicar una versión nueva, sube el número de Version.</t>
+          <t>6c. ReglasGenerales.Seccion: Gastos, Proyecto, Entrega o Cofinanciamiento. Define en qué parte de la guía aparece la regla.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>6d. En los textos puedes escribir [tu folio]: el programa lo reemplaza por el folio del proyecto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>8. Al publicar una versión nueva, sube el número de Version.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
           <t>9. Novedades: si la versión nueva cambia algo para los responsables, agrega en la hoja Novedades una fila por cambio, con el número de la versión nueva. El programa las muestra hasta que el responsable las marca como leídas.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Pendiente de validar</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
+    <row r="19">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>10. Programa y Descarga (filas de arriba): la última versión del programa (ej. 0.3.0) y el enlace https:// a su instalador. Si un programa instalado es más viejo, al abrirse avisa y muestra el enlace; si Descarga está vacía, pide el instalador al supervisor. Cámbialas solo cuando el instalador nuevo ya esté disponible en ese enlace.</t>
+        </is>
+      </c>
+    </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Cambios en la versión 4</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
-        </is>
-      </c>
+      <c r="B20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Pendiente de validar</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 5</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 4</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Cambios en la versión 3</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>

</xml_diff>

<commit_message>
Reglas v6 (23-10-2026): hojas Feriados (2026 a 2028), Topes y Glosario
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -16,8 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoFinanciables" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasGenerales" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plazos" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feriados" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topes" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Subitems'!$A$1:$F$29</definedName>
@@ -27,8 +30,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'NoFinanciables'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ReglasGenerales'!$A$1:$I$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Plazos'!$A$1:$J$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -473,7 +476,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2">
@@ -483,7 +486,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="3">
@@ -618,64 +621,97 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>11. Feriados: los feriados nacionales, para contar días hábiles (por ejemplo, el plazo de 15 días hábiles de cada rendición mensual). Agrega los del año siguiente antes de que empiece y los feriados por elecciones cuando se fijen. Los regionales no se cuentan (pregunta abierta a Jurídico).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Pendiente de validar</t>
-        </is>
-      </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
+          <t>12. Topes: el porcentaje máximo del monto pedido al fondo que puede sumar un subítem, según las bases de cada línea. El programa avisa si la postulación lo pasa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>13. Glosario: términos que el programa explica en pantalla y en la guía.</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Cambios en la versión 5</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
-        </is>
-      </c>
+      <c r="B23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Pendiente de validar</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Cambios en la versión 3</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
-        </is>
-      </c>
-    </row>
+          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Cambios en la versión 6</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 5</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 4</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -687,6 +723,1493 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>46023</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Año Nuevo</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Viernes Santo</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>46116</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Sábado Santo</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Día del Trabajo</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Glorias Navales</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Día Nacional de los Pueblos Indígenas</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Ley 21.357 (solsticio de invierno)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>San Pedro y San Pablo</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Virgen del Carmen</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Ley 20.148</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>46249</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Asunción de la Virgen</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Independencia Nacional</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>46284</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Glorias del Ejército</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Encuentro de Dos Mundos</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Iglesias Evangélicas y Protestantes</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Ley 20.299</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Día de Todos los Santos</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>46364</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Inmaculada Concepción</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>46381</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Navidad</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Año Nuevo</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>46472</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Viernes Santo</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>46473</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Sábado Santo</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>46508</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Día del Trabajo</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>46528</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Glorias Navales</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>46559</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Día Nacional de los Pueblos Indígenas</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Ley 21.357 (solsticio de invierno)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>46566</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>San Pedro y San Pablo</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Ley 19.668 (trasladado al lunes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>46584</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Virgen del Carmen</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Ley 20.148</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>46614</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Asunción de la Virgen</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>46647</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Feriado de Fiestas Patrias (17 de septiembre en viernes)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Ley 20.983</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>46648</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Independencia Nacional</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>46649</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Glorias del Ejército</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>46671</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Encuentro de Dos Mundos</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Ley 19.668 (trasladado al lunes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>46691</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Iglesias Evangélicas y Protestantes</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Ley 20.299</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>46692</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Día de Todos los Santos</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>46729</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Inmaculada Concepción</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>46746</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Navidad</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>46753</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Año Nuevo</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>46857</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Viernes Santo</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>46858</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Sábado Santo</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>46874</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Día del Trabajo</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>46894</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Glorias Navales</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
+        <v>46924</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Día Nacional de los Pueblos Indígenas</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Ley 21.357 (solsticio de invierno)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
+        <v>46930</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>San Pedro y San Pablo</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Ley 19.668 (trasladado al lunes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n">
+        <v>46950</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Virgen del Carmen</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Ley 20.148</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>46980</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Asunción de la Virgen</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>47014</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Independencia Nacional</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>47015</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Glorias del Ejército</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
+        <v>47035</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Encuentro de Dos Mundos</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Ley 19.668 (trasladado al lunes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>47053</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Día de las Iglesias Evangélicas y Protestantes</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Ley 20.299 (trasladado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n">
+        <v>47058</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Día de Todos los Santos</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n">
+        <v>47095</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Inmaculada Concepción</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n">
+        <v>47112</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Navidad</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Ley 2.977</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Subitem</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>VigenteDesde</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>VigenteHasta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Actividades Formativas</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Culturas Regionales</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Creación Artística</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Difusión</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Culturas Tradicionales</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Libro</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Fomento de la Lectura</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Bases Libro 2027 · Fomento de la Lectura, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Actividades Formativas</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Asignación del responsable</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Culturas Regionales</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Asignación del responsable</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Creación Artística</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Asignación del responsable</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Difusión</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Asignación del responsable</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Fondart Regional</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Culturas Tradicionales</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Asignación del responsable</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Bases Fondart Regional 2027, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Libro</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Fomento de la Lectura</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Asignación del responsable</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Bases Libro 2027 · Fomento de la Lectura, cap. I N°7</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G13" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Termino</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Explicacion</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Subítem</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>El tipo de gasto dentro de cada ítem del presupuesto (Personal, Operación o Inversión). De él depende qué documentos te piden para rendirlo.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. IV</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Verificador</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Una prueba de que una actividad se hizo: fotos con fecha, listas de asistencia firmadas, programas o registros audiovisuales. Cada actividad necesita al menos 3 distintos.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 1.02 N°3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Glosa</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>El texto que le pides al proveedor que escriba en la boleta o factura para dejar claro que el gasto es de tu proyecto.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. II</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SISREC</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>El Sistema de Rendición Electrónica de Cuentas de la Contraloría: ahí cargas tus gastos y tus informes.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 27</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Rendición sin movimiento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>La rendición que ingresas en SISREC en un mes en que no tuviste gastos.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3391, punto 5.3.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Días hábiles</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>De lunes a viernes, sin contar los feriados.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Ley 19.880, art. 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Total tramitación</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>El momento en que la resolución que aprueba tu convenio queda firmada y numerada. Desde ahí valen tus gastos.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 36</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Reitemización</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Mover dinero de un ítem del presupuesto a otro (por ejemplo, de Operación a Personal). Siempre requiere autorización y un anexo del convenio.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01; Memo 06/455</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Readecuación</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>El ajuste del presupuesto cuando te asignan menos de lo que pediste: dice cómo queda repartido el monto asignado.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Bases 2027, Anexo N°3, I N°5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Garantía</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>El documento que entregas para asegurar el buen uso de los recursos, por ejemplo una letra de cambio. Debe estar vigente hasta el cierre del convenio; la letra de cambio se renueva cada 6 meses.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 1.02 N°5; Memo 02/1264</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Prórroga</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Una extensión del plazo de ejecución del proyecto. Se pide antes de que venza el convenio, con al menos 30 días corridos de anticipación.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Glosario</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Cofinanciamiento</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Los aportes, tuyos o de terceros, que completan el costo del proyecto además de lo que pone el fondo.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. IV</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Informe de ejecución de actividades</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>El informe que cuenta qué actividades hiciste en el período, con sus verificadores. Con la Res. 2/2026 se entrega cada mes junto con el informe de rendición financiera, en el formato de la Contraloría (IN17).</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, arts. 24 y 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Supervisor</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>La persona de la SEREMI o del Ministerio que hace el seguimiento de tu convenio y responde tus consultas.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3095</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Fuerza mayor</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Un hecho que no podías prever ni evitar, como una catástrofe. Debes acreditarlo, y el Ministerio lo evalúa caso a caso.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1283</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Comprobante de pago</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>El documento que prueba que pagaste: transferencia, depósito, voucher de débito o recibo firmado.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. II</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -944,7 +2467,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Reglas v7: hoja Etapas («Así avanza tu proyecto»)
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -15,12 +15,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verificadores" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoFinanciables" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasGenerales" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plazos" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feriados" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topes" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etapas" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plazos" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feriados" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Subitems'!$A$1:$F$29</definedName>
@@ -29,9 +30,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Verificadores'!$A$1:$G$183</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'NoFinanciables'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ReglasGenerales'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Plazos'!$A$1:$J$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plazos'!$A$1:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -476,7 +477,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2">
@@ -546,7 +547,7 @@
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>3. VigenteDesde y VigenteHasta: rango de fechas de la resolución que aprueba el convenio en que aplica la regla. Vacío = sin límite.</t>
+          <t>3. VigenteDesde y VigenteHasta: rango de fechas de firma del convenio en que aplica la regla (si no se conoce la firma, se usa la fecha de la resolución que lo aprueba; Memo 02/580). Vacío = sin límite.</t>
         </is>
       </c>
     </row>
@@ -642,76 +643,95 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>14. Etapas: los textos de «Así avanza tu proyecto» en la guía, uno por fila. Orden 1 a 7 son las etapas y 8 el desvío «¿Necesitas cambiar algo?»; no cambies esos números, porque el programa pone las fechas del responsable en las etapas 2, 4 y 6 y en el desvío. Las filas con el mismo Orden llevan el mismo nombre en Etapa. Parte: Intro, Tú, Ministerio, Plazos u Ojo; dentro de cada etapa las partes salen en el orden de las filas. Lo que rige solo con la Res. 30/2015 lleva VigenteHasta 30-06-2026, y lo de la Res. 2/2026, VigenteDesde 01-07-2026.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Pendiente de validar</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Cambios en la versión 6</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
-        </is>
-      </c>
-    </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Cambios en la versión 4</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -723,6 +743,943 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Explicacion</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>VigenteDesde</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>VigenteHasta</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>PRORROGA_ANTICIPACION</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pedir una prórroga</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>días corridos</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Pide la prórroga al menos 30 días corridos antes de que venza el convenio.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Glosario (Prórroga)</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>MODIFICACION_ANTICIPACION</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Pedir una modificación</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Pide los cambios que necesitan autorización (fechas, equipo, mover dinero entre ítems) con 15 días hábiles de anticipación y espera la autorización antes de hacerlos.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>PRORROGA_MAXIMO</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Máximo de prórrogas</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>prórrogas</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Se aceptan hasta 2 prórrogas por atraso en las actividades. Una tercera es excepcional y, si eres institución privada, exige una caución de al menos el 5% del monto transferido.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°3</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>PRORROGA_EXTENSION_MAX</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Extensión máxima del plazo</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>% de la duración</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>El plazo puede extenderse como máximo un 50% de la duración original: un proyecto de 12 meses, hasta 18.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Art. V, Sección 5.01</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>GARANTIA_RENOVACION</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Renovar la letra de cambio</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>meses</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Si tu garantía es una letra de cambio, renuévala cada 6 meses desde su emisión. Debe estar vigente hasta que se tramite el cierre de tu convenio; si no la renuevas, pueden ponerle término.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1264 (24-12-2025)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>GRACIA_DOCUMENTOS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Documentos después del término</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>días</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Hasta 5 días después del término de la ejecución puedes obtener boletas, facturas o comprobantes de pago de gastos hechos dentro del período y contemplados en tu postulación. El instructivo no precisa si son días hábiles o corridos.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°3</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>INFORME_AVANCE_LARGO</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Informe de avance en proyectos largos</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>mes de ejecución</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Si tu proyecto dura más de 10 meses, debes presentar al menos un informe de avance al octavo mes.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3094, Firma de convenio N°5</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>INFORME_MENSUAL</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Informes mensuales</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>La norma de Contraloría pide entregar los informes financiero y de actividades dentro de los primeros 15 días hábiles de cada mes siguiente, incluso si ese mes no hubo gastos; si no, la cuenta se tiene por no rendida. Confirma con tu supervisor qué periodicidad fija tu convenio.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>OBS_FINANCIERAS</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Responder observaciones financieras</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Si el revisor observa un gasto, tienes 10 días hábiles para responder o entregar lo que falte. Si tu convenio se rige por la Res. 2/2026, este plazo vale cuando te observan hasta el 31-12-2026; desde 2027 rige el plazo de la Contraloría.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. III, Sección 3.03</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>OBS_ACTIVIDADES</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Responder observaciones de actividades</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Si te observan el informe de actividades, tienes 20 días hábiles para corregir. Si tu convenio se rige por la Res. 2/2026, este plazo vale cuando te observan hasta el 31-12-2026; desde 2027 rige el plazo de la Contraloría.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Flujos de trabajo</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>OBS_RES2_2027</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Responder observaciones en 2027</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Si te comunican observaciones durante 2027, tienes 40 días hábiles para responder o corregir.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>OBS_RES2_2028</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Responder observaciones en 2028</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Si te comunican observaciones durante 2028, tienes 30 días hábiles para responder o corregir.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H13" s="5" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>OBS_RES2</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Responder observaciones desde 2029</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Si te comunican observaciones desde el 01-01-2029, tienes 20 días hábiles para responder o corregir.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°4</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>AVISO_INCUMPLIMIENTO</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Corregir un aviso de incumplimiento</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Si recibes un aviso de incumplimiento, tienes 10 días hábiles para corregir. Si no corriges, recibes un segundo aviso con 10 días hábiles más; después el Ministerio puede poner término al convenio y enviar el caso al Consejo de Defensa del Estado.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3097, Acciones ante el incumplimiento</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>REVISION_MINISTERIO</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Revisión financiera del Ministerio</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>meses</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Desde que se aprueban tus actividades, el área de finanzas tiene hasta 3 meses para revisar tu rendición financiera. Si tu convenio se rige por la Res. 2/2026, este plazo vale hasta el 31-12-2026.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. VI</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>REVISION_RES2_2027</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Revisión del Ministerio en 2027</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>En 2027 el Ministerio tiene 80 días hábiles, desde que recibe tu rendición, para aprobarla u observarla; y 40 días hábiles, desde tu respuesta, para aprobarla o rechazarla.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°3 y N°5 y art. segundo transitorio</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>REVISION_RES2_2028</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Revisión del Ministerio en 2028</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>En 2028 el Ministerio tiene 70 días hábiles, desde que recibe tu rendición, para aprobarla u observarla; y 30 días hábiles, desde tu respuesta, para aprobarla o rechazarla.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°3 y N°5 y art. segundo transitorio</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>REVISION_RES2</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Revisión del Ministerio desde 2029</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Desde 2029 el Ministerio tiene 60 días hábiles, desde que recibe tu rendición, para aprobarla u observarla; y 20 días hábiles, desde tu respuesta, para aprobarla o rechazarla.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°3 y N°5</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H19" s="5" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>INFORME_FINAL_RES2</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Pronunciamiento sobre el informe final</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>meses</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Desde el término de las actividades, el Ministerio tiene hasta 6 meses para pronunciarse sobre tu informe final.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°6</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H20" s="5" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>CIERRE</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Cierre del convenio</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>días hábiles</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Aprobado el informe financiero final, el Ministerio tiene 60 días hábiles para dictar la resolución de cierre; luego te pide retirar tu garantía.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3097, Cierre N°6 y N°7</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="5" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1493,7 +2450,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1901,7 +2858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2209,7 +3166,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2467,7 +3424,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7615,7 +8572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7931,6 +8888,24 @@
       <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Memo 02/490</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en la guía: «Así avanza tu proyecto», las 7 etapas de tu convenio, desde que te seleccionan hasta el cierre: qué haces tú, qué hace el Ministerio, tus plazos y tus fechas en cada una.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3; Rex 3097</t>
         </is>
       </c>
     </row>
@@ -20934,45 +21909,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Clave</t>
+          <t>Orden</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Concepto</t>
+          <t>Etapa</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Cantidad</t>
+          <t>Parte</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Unidad</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Explicacion</t>
+          <t>TipoPersona</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -21002,36 +21977,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>PRORROGA_ANTICIPACION</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Pedir una prórroga</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>30</v>
+          <t>Te seleccionan</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Intro</t>
+        </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>días corridos</t>
+          <t>Tu proyecto fue seleccionado. Antes de firmar, el Ministerio necesita algunos documentos.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Pide la prórroga al menos 30 días corridos antes de que venza el convenio.</t>
+          <t>Todas</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.3, Glosario (Prórroga)</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
+          <t>Rex 3096, Instr. 4.3, Art. II</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21044,36 +22019,36 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>MODIFICACION_ANTICIPACION</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Pedir una modificación</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>15</v>
+          <t>Te seleccionan</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>días hábiles</t>
+          <t>Entrega la garantía que pide tu convenio, por ejemplo una letra de cambio: un documento en que te comprometes a devolver los recursos si no cumples.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pide los cambios que necesitan autorización (fechas, equipo, mover dinero entre ítems) con 15 días hábiles de anticipación y espera la autorización antes de hacerlos.</t>
+          <t>Todas</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.3, Sección 3.01</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+          <t>Rex 3096, Instr. 4.3, Art. I N°5</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21086,334 +22061,332 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>PRORROGA_MAXIMO</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Máximo de prórrogas</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
+          <t>Te seleccionan</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Entrega una copia de tu cédula de identidad.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Natural</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Art. II</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Te seleccionan</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Entrega una copia del RUT de tu organización.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Juridica</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Art. II</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Te seleccionan</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Inscribe a tu organización en el Registro de Personas Jurídicas Receptoras de Fondos Públicos (registros19862.cl), si todavía no lo está.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Juridica</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Ley 19.862</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Te seleccionan</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Revisa tus documentos y prepara tu convenio.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Art. II</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Te seleccionan</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Plazos</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Si tu garantía es una letra de cambio, renuévala cada 6 meses desde que se emitió y mantenla vigente hasta que se cierre tu convenio. Si no la renuevas, el Ministerio puede ponerle término a tu convenio.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1264</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>prórrogas</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Se aceptan hasta 2 prórrogas por atraso en las actividades. Una tercera es excepcional y, si eres institución privada, exige una caución de al menos el 5% del monto transferido.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°3</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>PRORROGA_EXTENSION_MAX</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Extensión máxima del plazo</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>% de la duración</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>El plazo puede extenderse como máximo un 50% de la duración original: un proyecto de 12 meses, hasta 18.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Art. V, Sección 5.01</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>GARANTIA_RENOVACION</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Renovar la letra de cambio</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>meses</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Si tu garantía es una letra de cambio, renuévala cada 6 meses desde su emisión. Debe estar vigente hasta que se tramite el cierre de tu convenio; si no la renuevas, pueden ponerle término.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Memo 02/1264 (24-12-2025)</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>GRACIA_DOCUMENTOS</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Documentos después del término</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>días</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Hasta 5 días después del término de la ejecución puedes obtener boletas, facturas o comprobantes de pago de gastos hechos dentro del período y contemplados en tu postulación. El instructivo no precisa si son días hábiles o corridos.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°3</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>INFORME_AVANCE_LARGO</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Informe de avance en proyectos largos</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>mes de ejecución</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Si tu proyecto dura más de 10 meses, debes presentar al menos un informe de avance al octavo mes.</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3094, Firma de convenio N°5</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Firmas el convenio</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Intro</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>El convenio es el acuerdo con el Ministerio: dice qué harás, cuánto puedes gastar y cuándo entregas tus informes.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujos de trabajo (línea de tiempo)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Firmas el convenio</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Lee tu convenio antes de firmarlo y guarda una copia: tus fechas de informes y tu presupuesto salen de ahí.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujos de trabajo (línea de tiempo)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Firmas el convenio</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Todavía no gastes. Espera a que la resolución que aprueba tu convenio quede totalmente tramitada, es decir, con todos sus trámites terminados. Pregúntale a tu supervisor desde qué fecha lo está.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Res. 30/2015 CGR, art. 13</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="5" t="n">
         <v>46203</v>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>INFORME_MENSUAL</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Informes mensuales</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>días hábiles</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>La norma de Contraloría pide entregar los informes financiero y de actividades dentro de los primeros 15 días hábiles de cada mes siguiente, incluso si ese mes no hubo gastos; si no, la cuenta se tiene por no rendida. Confirma con tu supervisor qué periodicidad fija tu convenio.</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Res. 2/2026 CGR, art. 25 N°2</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>46204</v>
-      </c>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>OBS_FINANCIERAS</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Responder observaciones financieras</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>días hábiles</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Si el revisor observa un gasto, tienes 10 días hábiles para responder o entregar lo que falte. Si tu convenio se rige por la Res. 2/2026, este plazo vale cuando te observan hasta el 31-12-2026; desde 2027 rige el plazo de la Contraloría.</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.2, Art. III, Sección 3.03</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>OBS_ACTIVIDADES</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Responder observaciones de actividades</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>días hábiles</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Si te observan el informe de actividades, tienes 20 días hábiles para corregir. Si tu convenio se rige por la Res. 2/2026, este plazo vale cuando te observan hasta el 31-12-2026; desde 2027 rige el plazo de la Contraloría.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.1, Flujos de trabajo</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21426,38 +22399,38 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>OBS_RES2_2027</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Responder observaciones en 2027</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>40</v>
+          <t>Firmas el convenio</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>días hábiles</t>
+          <t>Todavía no gastes. Espera a que la resolución que aprueba tu convenio quede totalmente tramitada, es decir, con todos sus trámites terminados. Pregúntale a tu supervisor desde qué fecha lo está.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Si te comunican observaciones durante 2027, tienes 40 días hábiles para responder o corregir.</t>
+          <t>Todas</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio</t>
+          <t>Res. 2/2026 CGR, art. 36</t>
         </is>
       </c>
       <c r="G12" s="5" t="n">
         <v>46204</v>
       </c>
-      <c r="H12" s="5" t="n"/>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21470,124 +22443,124 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>OBS_RES2_2028</t>
-        </is>
+      <c r="A13" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Responder observaciones en 2028</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>30</v>
+          <t>Firmas el convenio</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>días hábiles</t>
+          <t>Firma el convenio y dicta la resolución que lo aprueba.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Si te comunican observaciones durante 2028, tienes 30 días hábiles para responder o corregir.</t>
+          <t>Todas</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n">
+          <t>Rex 3096, Instr. 4.3, Flujos de trabajo (línea de tiempo)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Firmas el convenio</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Ojo</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Los gastos hechos antes de la total tramitación no se aceptan, salvo que tu convenio y la resolución que lo aprueba los autoricen expresamente por razones de continuidad o buen servicio.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Res. 30/2015 CGR, art. 13; Memo 06/561</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Firmas el convenio</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Ojo</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Los gastos hechos antes de la total tramitación no se aceptan, salvo que tu convenio y la resolución que lo aprueba los autoricen expresamente por razones de continuidad o buen servicio.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 36; Memo 06/561</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
         <v>46204</v>
       </c>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>OBS_RES2</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Responder observaciones desde 2029</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>días hábiles</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Si te comunican observaciones desde el 01-01-2029, tienes 20 días hábiles para responder o corregir.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Res. 2/2026 CGR, art. 25 N°4</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>46204</v>
-      </c>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>AVISO_INCUMPLIMIENTO</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Corregir un aviso de incumplimiento</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>días hábiles</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Si recibes un aviso de incumplimiento, tienes 10 días hábiles para corregir. Si no corriges, recibes un segundo aviso con 10 días hábiles más; después el Ministerio puede poner término al convenio y enviar el caso al Consejo de Defensa del Estado.</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3097, Acciones ante el incumplimiento</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
+      <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21600,80 +22573,78 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>REVISION_MINISTERIO</t>
-        </is>
+      <c r="A16" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Revisión financiera del Ministerio</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
+          <t>Recibes los recursos</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Cuando recibas la transferencia, firma el comprobante de ingreso que te envía el Ministerio y devuélvelo. Es la prueba de que recibiste los recursos.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3094, Sección 4.01 N°4</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>meses</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Desde que se aprueban tus actividades, el área de finanzas tiene hasta 3 meses para revisar tu rendición financiera. Si tu convenio se rige por la Res. 2/2026, este plazo vale hasta el 31-12-2026.</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3096, Instr. 4.2, Art. VI</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>REVISION_RES2_2027</t>
-        </is>
-      </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Revisión del Ministerio en 2027</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>80</v>
+          <t>Recibes los recursos</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>días hábiles</t>
+          <t>Usa los recursos solo en lo que te aprobaron para tu proyecto.</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>En 2027 el Ministerio tiene 80 días hábiles, desde que recibe tu rendición, para aprobarla u observarla; y 40 días hábiles, desde tu respuesta, para aprobarla o rechazarla.</t>
+          <t>Todas</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Res. 2/2026 CGR, art. 25 N°3 y N°5 y art. segundo transitorio</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>46204</v>
-      </c>
-      <c r="H17" s="5" t="n"/>
+          <t>Rex 3096, Instr. 4.3, Art. II</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21686,38 +22657,38 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>REVISION_RES2_2028</t>
-        </is>
+      <c r="A18" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Revisión del Ministerio en 2028</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>70</v>
+          <t>Recibes los recursos</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>días hábiles</t>
+          <t>Te transfiere los recursos como indica tu convenio: de una vez o en cuotas.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>En 2028 el Ministerio tiene 70 días hábiles, desde que recibe tu rendición, para aprobarla u observarla; y 30 días hábiles, desde tu respuesta, para aprobarla o rechazarla.</t>
+          <t>Todas</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Res. 2/2026 CGR, art. 25 N°3 y N°5 y art. segundo transitorio</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>46204</v>
-      </c>
-      <c r="H18" s="5" t="n"/>
+          <t>Res. 30/2015 CGR, art. 19</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="5" t="n">
+        <v>46203</v>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21730,38 +22701,38 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>REVISION_RES2</t>
-        </is>
+      <c r="A19" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Revisión del Ministerio desde 2029</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>60</v>
+          <t>Recibes los recursos</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>días hábiles</t>
+          <t>Te transfiere los recursos como indica tu convenio. En 2026, a los beneficiarios de los Fondos se les paga en una sola cuota.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Desde 2029 el Ministerio tiene 60 días hábiles, desde que recibe tu rendición, para aprobarla u observarla; y 20 días hábiles, desde tu respuesta, para aprobarla o rechazarla.</t>
+          <t>Todas</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Res. 2/2026 CGR, art. 25 N°3 y N°5</t>
+          <t>Res. 2/2026 CGR, art. 25 N°1; Memo 02/064; Dictamen CGR OF192150</t>
         </is>
       </c>
       <c r="G19" s="5" t="n">
         <v>46204</v>
       </c>
-      <c r="H19" s="5" t="n"/>
+      <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Todos</t>
@@ -21774,93 +22745,1854 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>INFORME_FINAL_RES2</t>
-        </is>
+      <c r="A20" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Pronunciamiento sobre el informe final</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Intro</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Mientras haces tus actividades, vas mostrando qué hiciste y en qué gastaste.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujo general del proyecto</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Junta los documentos de cada gasto y los verificadores de cada actividad a medida que avanzas, no al final. Los checklists de esta guía te dicen cuáles.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujo general del proyecto</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Cada informe tiene dos partes: el de actividades (qué hiciste, con fotos, listas de asistencia y otros verificadores) y el financiero (en qué gastaste, con boletas, facturas y comprobantes de pago).</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujo general del proyecto</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Entrega tus informes de avance en las fechas de tu convenio.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Tu convenio; Res. 30/2015 CGR, art. 27</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Si tu proyecto dura más de 10 meses, entrega al menos un informe de avance cerca del octavo mes.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3094, Firma de convenio N°5</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Si tu convenio no fija fechas, entrega un informe cada mes, dentro de los primeros 15 días hábiles del mes siguiente.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Res. 30/2015 CGR, art. 27 a)</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Revisa en tu convenio si rindes en SISREC, la plataforma en línea de la Contraloría, o en papel: con esta norma, los convenios de menos de 500 UTM pueden rendir en papel.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/872</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Cada mes entrega juntos el informe de actividades y el financiero, dentro de los primeros 15 días hábiles del mes siguiente.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°2; Memo 02/566, punto III</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Entrégalos aunque ese mes no hayas gastado ni hecho actividades: es la rendición «sin movimiento». Si no los entregas, se considera que no rendiste cuentas.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°2; Rex 3391, punto 5.3.1</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Rinde en SISREC, la plataforma en línea de la Contraloría para rendir cuentas.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 27; Memo 02/566, punto V</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H29" s="2" t="n"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Haces tu proyecto y rindes</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Ojo</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Mientras tengas una rendición vencida sin entregar, el Ministerio no puede entregarte recursos de otros convenios. Basta con que la entregues: no hace falta que ya esté aprobada.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Res. 30/2015 CGR, art. 18; Res. 2/2026 CGR, art. 38; Memo 02/978</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Intro</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>El Ministerio revisa cada informe para comprobar que hiciste lo que comprometiste y que tus gastos están bien respaldados.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujo general del proyecto</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Tu supervisor revisa primero las actividades. Si las aprueba, el informe pasa a un revisor financiero, que revisa los gastos.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujo general del proyecto</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Si todo está bien, te envía un certificado de aprobación (estado «Sigue»). Si falta algo, te envía un informe de observaciones con lo que debes corregir (estado «Debes corregir»).</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Flujos de trabajo</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Al terminar, recibes un certificado de aprobación total o, si quedó algo sin aprobar, uno de aprobación parcial que dice qué monto debes justificar o devolver.</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Anexos 1 y 2</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Lee las observaciones con calma y responde dentro del plazo, con los documentos que faltan o una explicación, por el medio que te indiquen.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Sección 3.03</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Si tienes dudas, consulta a tu supervisor antes de que venza el plazo.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Sección 3.03</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Plazos</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Para corregir tienes 20 días hábiles si te observan las actividades y 10 días hábiles si te observan gastos, contados desde que te avisan.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1, Flujos de trabajo; Instr. 4.2, Sección 3.03</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Plazos</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Para corregir, el plazo depende de cuándo te avisan las observaciones: hasta el 31-12-2026, 20 días hábiles (actividades) o 10 (gastos); durante 2027, 40 días hábiles; durante 2028, 30; desde 2029, 20.</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio; Rex 3096, Instr. 4.1 y 4.2</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H38" s="2" t="n"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Plazos</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Desde que aprueba tus actividades, el Ministerio tiene hasta 3 meses para revisar tus gastos.</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. VI</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n"/>
+      <c r="H39" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Plazos</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Hasta el 31-12-2026, el Ministerio tiene hasta 3 meses para revisar tus gastos desde que aprueba tus actividades. Desde 2027 tiene 80 días hábiles en 2027, 70 en 2028 y 60 desde 2029, contados desde que recibe tu rendición, para aprobarla u observarla. Después de tu respuesta, tiene 40, 30 o 20 días hábiles para aprobarla o rechazarla.</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°3 y N°5 y art. segundo transitorio; Rex 3096, Instr. 4.2, Art. VI</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Ojo</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Si no corriges, recibes un aviso de incumplimiento con 10 días hábiles para corregir. Si sigues sin hacerlo, recibes un segundo aviso con 10 días hábiles más.</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3097, Acciones ante el incumplimiento</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Ojo</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Si aun así no corriges, el Ministerio puede poner término a tu convenio, pedirte que devuelvas los recursos y enviar tu caso al Consejo de Defensa del Estado, que puede cobrarlos judicialmente.</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3097, Acciones ante el incumplimiento</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Te revisan</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Ojo</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Si un gasto no se puede justificar, te pedirán devolver ese monto. A esto se le llama reintegro.</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. VII</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>meses</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Desde el término de las actividades, el Ministerio tiene hasta 6 meses para pronunciarse sobre tu informe final.</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Entregas el informe final</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Al terminar tu proyecto, entrega el informe final de actividades y el financiero en la fecha que fija tu convenio.</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Res. 30/2015 CGR, art. 27</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Entregas el informe final</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Al terminar tu proyecto, entrega el informe final de actividades y el financiero en la fecha que fija tu convenio.</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°1</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Entregas el informe final</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Tienes hasta 5 días después del término de la ejecución para conseguir boletas o comprobantes de pago de gastos que ya hiciste.</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°3</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Entregas el informe final</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>El informe final se suma a los informes mensuales; no los reemplaza.</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°1 y N°2</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H47" s="2" t="n"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Entregas el informe final</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Revisa el informe final igual que los anteriores: primero las actividades y después los gastos. Los plazos para corregir son los de la etapa 5.</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Flujo general del proyecto</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Entregas el informe final</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Tiene hasta 6 meses, desde el término de tus actividades, para pronunciarse sobre tu informe final.</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Res. 2/2026 CGR, art. 25 N°6</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="G49" s="5" t="n">
         <v>46204</v>
       </c>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>Todas</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>CIERRE</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Cierre del convenio</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>días hábiles</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Aprobado el informe financiero final, el Ministerio tiene 60 días hábiles para dictar la resolución de cierre; luego te pide retirar tu garantía.</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Rex 3097, Cierre N°6 y N°7</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Todos</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="H49" s="2" t="n"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Se cierra tu convenio</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Cuando aprueba tu informe financiero final, tiene 60 días hábiles para dictar la resolución que cierra tu convenio. A esto se le llama cierre administrativo.</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3097, Cierre del convenio N°6</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n"/>
+      <c r="H50" s="2" t="n"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Se cierra tu convenio</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Te avisa del cierre y te pide retirar tu garantía.</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3097, Cierre del convenio N°7</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n"/>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Se cierra tu convenio</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Si te pidieron devolver dinero, hazlo en el plazo que indique tu convenio y guarda el comprobante.</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Tu convenio</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Se cierra tu convenio</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Si te pidieron devolver dinero, hazlo en el plazo que indique tu convenio y guarda el comprobante.</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Tu convenio; Res. 2/2026 CGR, art. 26 N°6</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Se cierra tu convenio</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Retira tu garantía cuando te avisen del cierre.</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3097, Cierre del convenio N°7</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n"/>
+      <c r="H54" s="2" t="n"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Intro</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Puedes pedir cambios, pero siempre antes de hacerlos.</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n"/>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Pide el cambio antes de hacerlo y no lo hagas hasta que te lo autoricen por escrito.</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n"/>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Cambios menores, como mover la fecha o el lugar de una actividad dentro del plazo del convenio: pídelos con 15 días hábiles de anticipación y explica por qué. Para ajustar gastos dentro de un mismo ítem, revisa la cláusula de modificaciones de tu convenio.</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°1; Memo 06/455</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Cambios mayores, como cambiar a alguien del equipo, mover dinero de un ítem a otro (a esto se le llama reitemización) o cambiar la fecha del informe final: pídelos con el anexo de solicitud de tu convenio, con 15 días hábiles de anticipación y con los documentos que los respalden.</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°2; Memo 06/455</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n"/>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Prórroga (más plazo para tu proyecto): pídela al menos 30 días corridos antes de que venza tu convenio, con un nuevo cronograma y un informe de lo que llevas hecho. Se aceptan hasta 2 prórrogas, y el plazo total puede crecer como máximo la mitad de lo que dura tu proyecto. Si te la aprueban, renueva tu garantía para que cubra el nuevo plazo.</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Glosario (Prórroga), Sección 3.01 N°3 y Sección 5.01</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n"/>
+      <c r="H59" s="2" t="n"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Tú</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Una tercera prórroga solo se da en casos excepcionales y exige una garantía adicional de al menos el 5% del monto transferido.</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Juridica</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3094, Art. V N°1 y N°3</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n"/>
+      <c r="H60" s="2" t="n"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Evalúa tu solicitud. Si la aprueba, dicta una resolución exenta (el acto formal que la autoriza). Si no, te responde con un oficio (una carta formal) que la rechaza.</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 (flujo de gestión de modificación sustantiva)</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n"/>
+      <c r="H61" s="2" t="n"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>¿Necesitas cambiar algo de tu proyecto?</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>No tiene un plazo fijo para responder; por eso conviene pedir con anticipación.</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n"/>
+      <c r="H62" s="2" t="n"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
         <is>
           <t>Todas</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J15"/>
+  <dataValidations count="2">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Intro,Tú,Ministerio,Plazos,Ojo"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Todas,Natural,Juridica"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Reglas v8: novedades según la versión del programa; programa 0.3.1-prueba
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -498,7 +498,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.2.0-prueba</t>
+          <t>0.3.1-prueba</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>9. Novedades: si la versión nueva cambia algo para los responsables, agrega en la hoja Novedades una fila por cambio, con el número de la versión nueva. El programa las muestra hasta que el responsable las marca como leídas.</t>
+          <t>9. Novedades: si la versión nueva cambia algo para los responsables, agrega en la hoja Novedades una fila por cambio, con el número de la versión nueva. El programa las muestra hasta que el responsable las marca como leídas. Si la novedad anuncia algo que solo trae un programa nuevo, escribe en DesdePrograma la versión que lo trae (ej. 0.3.1-prueba): los programas anteriores no la muestran. Vacío = la ven todos.</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>14. Etapas: los textos de «Así avanza tu proyecto» en la guía, uno por fila. Orden 1 a 7 son las etapas y 8 el desvío «¿Necesitas cambiar algo?»; no cambies esos números, porque el programa pone las fechas del responsable en las etapas 2, 4 y 6 y en el desvío. Las filas con el mismo Orden llevan el mismo nombre en Etapa. Parte: Intro, Tú, Ministerio, Plazos u Ojo; dentro de cada etapa las partes salen en el orden de las filas. Lo que rige solo con la Res. 30/2015 lleva VigenteHasta 30-06-2026, y lo de la Res. 2/2026, VigenteDesde 01-07-2026.</t>
+          <t>14. Etapas: los textos de «Así avanza tu proyecto» en la guía, uno por fila. Orden 1 a 7 son las etapas y 8 el desvío «¿Necesitas cambiar algo?»; no cambies esos números, porque el programa pone las fechas del responsable en las etapas 1, 2, 4 y 6 y en el desvío. Las filas con el mismo Orden llevan el mismo nombre en Etapa. Parte: Intro, Tú, Ministerio, Plazos u Ojo; dentro de cada etapa las partes salen en el orden de las filas. Lo que rige solo con la Res. 30/2015 lleva VigenteHasta 30-06-2026, y lo de la Res. 2/2026, VigenteDesde 01-07-2026.</t>
         </is>
       </c>
     </row>
@@ -664,74 +664,85 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 4</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -8572,13 +8583,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="95" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8602,6 +8614,11 @@
           <t>Fuente</t>
         </is>
       </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>DesdePrograma</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -8620,6 +8637,7 @@
           <t>Memo 02/566, punto V</t>
         </is>
       </c>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -8638,6 +8656,7 @@
           <t>Res. 2/2026 CGR, art. 38; Memo 02/566, punto IV</t>
         </is>
       </c>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -8656,6 +8675,7 @@
           <t>Memo 02/1264</t>
         </is>
       </c>
+      <c r="E4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -8674,6 +8694,7 @@
           <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio</t>
         </is>
       </c>
+      <c r="E5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -8692,6 +8713,7 @@
           <t>Rex 3391, Anexo A</t>
         </is>
       </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -8710,6 +8732,7 @@
           <t>Rex 3391, Anexo A letra d)</t>
         </is>
       </c>
+      <c r="E7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -8728,6 +8751,7 @@
           <t>Rex 3096; Rex 3391, Anexo A letra j)</t>
         </is>
       </c>
+      <c r="E8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -8746,6 +8770,7 @@
           <t>Memo 02/064; Dictamen CGR OF192150</t>
         </is>
       </c>
+      <c r="E9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -8764,6 +8789,7 @@
           <t>Rex 3390</t>
         </is>
       </c>
+      <c r="E10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -8782,6 +8808,7 @@
           <t>Bases de la Convocatoria 2027, tanda 1</t>
         </is>
       </c>
+      <c r="E11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -8800,6 +8827,7 @@
           <t>Memo 02/872</t>
         </is>
       </c>
+      <c r="E12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -8818,6 +8846,7 @@
           <t>Memo 02/978</t>
         </is>
       </c>
+      <c r="E13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -8836,6 +8865,7 @@
           <t>Memo 06/455</t>
         </is>
       </c>
+      <c r="E14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -8854,6 +8884,7 @@
           <t>Memo 06/561</t>
         </is>
       </c>
+      <c r="E15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -8872,6 +8903,7 @@
           <t>Memo 02/1283; Dictámenes CGR 16.096, 19.889 y 85.710</t>
         </is>
       </c>
+      <c r="E16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -8890,6 +8922,7 @@
           <t>Memo 02/490</t>
         </is>
       </c>
+      <c r="E17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -8906,6 +8939,34 @@
       <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Rex 3096, Instr. 4.3; Rex 3097</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>0.3.1-prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en el calendario de tu guía: las fechas para renovar tu garantía y, si tu convenio se rige por la Res. 2/2026, el plazo del Ministerio para pronunciarse sobre tu informe final.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1264; Res. 2/2026 CGR, art. 25 N°6</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>0.3.1-prueba</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reglas v9: programa 0.4.0-prueba
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
@@ -498,7 +498,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.3.1-prueba</t>
+          <t>0.4.0-prueba</t>
         </is>
       </c>
     </row>
@@ -664,85 +664,98 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cambios en la versión 8</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 4</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -8583,7 +8596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8967,6 +8980,25 @@
       <c r="E19" s="2" t="inlineStr">
         <is>
           <t>0.3.1-prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en el programa: tu proyecto queda guardado y lo retomas al abrirlo. «Tu próximo paso» te dice qué hacer ahora, y en «Mis gastos y documentos» y «Mis actividades» marcas cada documento y verificador como «lo tengo», «me falta» o «no aplica».</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>0.4.0-prueba</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reglas v10: Situaciones y SISREC; programa 0.5.0-prueba
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -16,12 +16,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NoFinanciables" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasGenerales" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etapas" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plazos" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feriados" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topes" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Situaciones" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SISREC" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plazos" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feriados" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Topes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Subitems'!$A$1:$F$29</definedName>
@@ -30,9 +32,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Verificadores'!$A$1:$G$183</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'NoFinanciables'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ReglasGenerales'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plazos'!$A$1:$J$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Plazos'!$A$1:$J$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'ErroresFrecuentes'!$A$1:$C$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'ReglasBases'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -477,7 +479,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2">
@@ -498,7 +500,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.4.0-prueba</t>
+          <t>0.5.0-prueba</t>
         </is>
       </c>
     </row>
@@ -650,112 +652,138 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>15. Situaciones: «¿Qué hago si…?». Una fila por situación (o una por norma o tipo de persona, si cambia): qué hacer, el plazo y quién firma (estos dos pueden ir vacíos). Las filas con el mismo nombre se muestran juntas; en los textos puedes escribir [tu folio].</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Pendiente de validar</t>
-        </is>
-      </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
+          <t>16. SISREC: un paso por fila, numerados desde 1 en cada trámite. En la fila del paso 1 va el enlace https:// al manual de la Contraloría.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr"/>
+    </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cambios en la versión 9</t>
+          <t>Pendiente de validar</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Cambios en la versión 8</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
-        </is>
-      </c>
-    </row>
+          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 10</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Cambios en la versión 5</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 4</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -767,6 +795,1671 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Situacion</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>QueHacer</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Plazo</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>QuienFirma</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>TipoPersona</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>VigenteDesde</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>VigenteHasta</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Necesito más plazo para terminar mis actividades</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Pide una prórroga con el formulario o anexo que viene con la resolución de tu convenio. Explica qué te impidió avanzar y adjunta un nuevo cronograma, cartas de compromiso (espacios, personas, imprentas) y un informe de lo que llevas hecho. Si te la aprueban, extiende tu garantía para que cubra el nuevo plazo.</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Al menos 30 días corridos antes de que venza tu convenio. Se aceptan hasta 2 prórrogas, y el plazo total puede crecer como máximo la mitad de lo que dura tu proyecto. Si tu garantía es una letra de cambio, entrega la nueva dentro de 2 días desde que te notifican la aprobación.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Tú, como responsable del proyecto; en una organización, su representante legal.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°3 y Glosario (Prórroga); Rex 1523/2024, art. primero N°2</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Necesito más plazo para terminar mis actividades</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Una tercera prórroga solo se da en casos excepcionales, con un informe técnico del Ministerio, y tu organización debe entregar una caución de al menos el 5% del monto transferido por el tiempo que se extiende.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tú, como responsable del proyecto; en una organización, su representante legal.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Juridica</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°3</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Terminé las actividades, pero necesito más tiempo para el informe final</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Pide ampliar el plazo de entrega del informe final. Indica que las actividades ya se hicieron dentro del plazo y adjunta el informe final de actividades con sus verificadores. Extiende también tu garantía.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Con 15 días hábiles de anticipación a la fecha de entrega que fija tu convenio.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Tú, como responsable del proyecto; en una organización, su representante legal.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°2 y N°3</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Quiero mover dinero o cambiar un gasto</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Mover dinero de un ítem a otro (reitemización) siempre necesita autorización previa y un anexo del convenio: explica por qué y adjunta cotizaciones o compromisos. Dentro de un mismo ítem, revisa la cláusula de modificaciones de tu convenio; si no lo permite, o si se trata de alojamiento, alimentación o traslado, pide autorización. Tu asignación como responsable nunca puede subir. No hagas el gasto hasta que te autoricen por escrito.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Con 15 días hábiles de anticipación al gasto.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Tú, como responsable del proyecto; en una organización, su representante legal.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°1, N°2 y N°4; Memo 06/455</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Quiero cambiar la fecha o el lugar de una actividad</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Si la nueva fecha queda dentro del plazo de tu convenio, es un cambio menor: avísalo y explica por qué. Un cambio de lugar lo evalúa tu supervisor, que puede considerarlo un cambio mayor. Si la actividad queda fuera del plazo de tu convenio, necesitas una prórroga.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Con 15 días hábiles de anticipación.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Tú, como responsable del proyecto; en una organización, su representante legal.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°1</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Necesito cambiar a alguien del equipo</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Es un cambio mayor: pídelo antes de hacerlo, con la carta de renuncia de quien se va, los pagos de lo que alcanzó a trabajar, el currículum de quien llega y su carta de compromiso con las funciones.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Con 15 días hábiles de anticipación al cambio.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Tú, como responsable del proyecto; en una organización, su representante legal.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.3, Sección 3.01 N°2 y N°5</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Tengo un gasto que no estaba en mi postulación</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>No lo hagas todavía: solo valen los gastos de tu presupuesto aprobado que se relacionan directamente con las actividades del proyecto. Si lo necesitas, pide autorización para mover dinero a ese gasto y espera la respuesta por escrito.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Con 15 días hábiles de anticipación.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Tú, como responsable del proyecto; en una organización, su representante legal.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. III, Sección 3.02; Instr. 4.3, Sección 3.01</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Me observaron un gasto o una actividad</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Lee la observación: en SISREC aparece como comentario en cada gasto «Rendida observada». Corrige los datos, entrega el documento que falta o explica lo que pasó, y vuelve a enviar la rendición. Si un gasto no se puede justificar, te pedirán devolver ese monto. Si tienes dudas, consulta a tu supervisor antes de que venza el plazo.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>20 días hábiles si te observan las actividades y 10 si te observan gastos, contados desde que te avisan.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>En SISREC, quien firma tus rendiciones (el encargado ejecutor), con su firma electrónica.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.1 (Flujos de trabajo) e Instr. 4.2 (Sección 3.03); Manual SISREC Ejecutor 07 (CGR)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="5" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Me observaron un gasto o una actividad</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Lee la observación: en SISREC aparece como comentario en cada gasto «Rendida observada». Corrige los datos, entrega el documento que falta o explica lo que pasó, y vuelve a enviar la rendición. Si un gasto no se puede justificar, te pedirán devolver ese monto. Si tienes dudas, consulta a tu supervisor antes de que venza el plazo.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Depende de cuándo te avisan: hasta el 31-12-2026, 20 días hábiles (actividades) o 10 (gastos); durante 2027, 40 días hábiles; durante 2028, 30; desde 2029, 20.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>En SISREC, quien firma tus rendiciones (el encargado ejecutor), con su firma electrónica.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°4 y art. segundo transitorio; Manual SISREC Ejecutor 07 (CGR)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Se me pasó la fecha de una rendición</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Entrégala cuanto antes y avísale a tu supervisor. Mientras tengas una rendición vencida sin entregar, el Ministerio no puede entregarte recursos de otros convenios, y puedes recibir un aviso de incumplimiento.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Después de un aviso de incumplimiento tienes 10 días hábiles para ponerte al día, y 10 más si recibes un segundo aviso. Después, el Ministerio puede poner término a tu convenio.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Res. 30/2015 CGR, art. 18; Res. 2/2026 CGR, art. 38; Rex 3097, Acciones ante el incumplimiento</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Se me pasó la fecha de una rendición</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Con la Res. 2/2026, si no entregas la rendición de un mes, se considera que no rendiste cuentas.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Perdí un documento</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Avisa de inmediato a tu supervisor y pide un duplicado al proveedor. Solo en casos especiales, que decide el Ministerio, se acepta otra prueba en vez del documento original.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>De inmediato, antes de rendir ese gasto.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Dictámenes CGR N° 19.889 de 2012 y 90.073 de 2016</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>El proveedor no puso la glosa en la boleta o factura</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Pide la glosa «Proyecto financiado por el MINCAP, Folio [tu folio]» antes de que te emitan el documento. Si el proveedor no puede ponerla, guarda el correo o mensaje donde se la pediste y preséntalo junto con el gasto.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2, Art. II y Art. VII</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Pagué con tarjeta de crédito</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Paga con débito, transferencia o efectivo. La tarjeta de crédito se acepta solo en casos excepcionales (por ejemplo, para no llevar efectivo en el extranjero); entonces rinde el voucher, la boleta o factura y el estado de cuenta pagado. Los intereses de pagar en cuotas no se financian.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen CGR N° 16.096 de 2017</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>No alcancé a gastar todo</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Lo que no gastaste, y lo que te rechacen, debes devolverlo al Ministerio (reintegro) y guardar el comprobante. Antes de cerrar el proyecto en SISREC tienes que haberlo devuelto, porque solo se cierran los proyectos sin saldo pendiente.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>En el plazo que fije tu convenio.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Tu convenio; Rex 3097, Cierre del convenio; Manual SISREC Ejecutor 11 (CGR)</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Un temporal, incendio o catástrofe me impide ejecutar</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Si un hecho que no podías prever ni evitar (un temporal, un incendio, una catástrofe declarada en tu región) te impide ejecutar, avisa a tu supervisor y acredítalo con documentos: el Ministerio lo evalúa caso a caso. Si la actividad se suspende, se hace en una nueva fecha con una prórroga y los mayores costos son tuyos; si se cancela, se pone término al convenio: rindes lo ya gastado y devuelves lo que no alcanzaste a usar. En julio de 2026, por ejemplo, La Araucanía y otras regiones fueron declaradas zona afectada por catástrofe.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Avísale a tu supervisor apenas ocurra.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Memo 02/1283 (25-11-2019); Memo 02/139 (10-02-2023); Decreto N° 113 de 2026 (Interior)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Todas,Natural,Juridica"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Tramite</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Paso</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Enlace</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Entrar a SISREC y dejar lista tu cuenta</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Entra a www.rendicioncuentas.cl/portal/sitiosisrec y presiona «Ingresar aquí». Inicias sesión con tu RUT y tu Clave Única.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/1._Manual_de_Administrador_del_SISREC_Ejecutor.pdf/38415c08-57d3-5dcc-1c96-e48297fd1cee</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 01 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Entrar a SISREC y dejar lista tu cuenta</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>En SISREC cada persona tiene un rol: el analista ejecutor carga las rendiciones, el ministro de fe compara lo escaneado con los documentos originales y el encargado ejecutor las firma y las envía al Ministerio. Si no sabes quién cumple cada rol en tu proyecto, pregúntale a tu supervisor.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 01 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Entrar a SISREC y dejar lista tu cuenta</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>El administrador de tu cuenta crea los usuarios y les asigna su rol en el menú «Administración» › «Usuarios».</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 01 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Entrar a SISREC y dejar lista tu cuenta</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Registra en «Administración» › «Cuentas bancarias» la cuenta donde recibirás los recursos: sin ella, el Ministerio no puede enviarte la transferencia.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 01 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Aceptar la transferencia</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Entra a SISREC y ve al menú «Transferencia» › «Mis ingresos».</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/3._Manual_Ejecutor_Aceptacion_o_rechazo_de_Transferencia.pdf/69905a76-8959-bfe3-7768-b3c824077ba1</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Aceptar la transferencia</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Busca la transferencia que te envió el Ministerio y ábrela con la lupa («Ver ingreso»).</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Aceptar la transferencia</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>En «Documentación complementaria» revisa lo que adjuntó el Ministerio: el comprobante de egreso, la cartola y la resolución que aprueba tu convenio. Presiona «Cerrar».</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Aceptar la transferencia</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>En «Estado» elige «Aceptar» y presiona «Nuevo» para agregar tu comprobante de ingreso.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Aceptar la transferencia</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Completa el nombre, el número y la fecha de la transferencia, adjunta el comprobante de ingreso y presiona «Guardar».</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Aceptar la transferencia</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Presiona «Aceptar». Desde el mes siguiente a la aceptación rindes cada mes.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Aceptar la transferencia</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Si algo no corresponde (el monto o el proyecto), elige «Rechazada», explica el motivo en «Comentario del rechazo» y avísale a tu supervisor.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Ingresar un proveedor</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Ingresa cada proveedor antes de rendir sus gastos: menú «Proveedores», botón «Nuevo».</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/2._Manual_Ejecutor_Ingreso_de_un_Proveedor.pdf/e6fc195a-c703-91a8-e5ed-b7ae3229aa1a</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 02 (CGR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Ingresar un proveedor</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Elige si es «Persona natural» o «Persona jurídica».</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 02 (CGR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Ingresar un proveedor</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Persona natural: escribe su RUN y SISREC trae su nombre desde el Registro Civil. Completa los demás campos.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 02 (CGR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Ingresar un proveedor</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Persona jurídica: escribe su RUT, su razón social y su giro.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 02 (CGR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Ingresar un proveedor</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Presiona «Guardar». También puedes agregarlo mientras rindes, con el botón «+» de la pantalla «Documento».</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 02 (CGR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Ve a «Rendiciones» › «Mis rendiciones» y presiona «Nuevo».</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/5._Manual_Ejecutor_Rendicion_Mensual.pdf/003c9e08-83a5-07c4-618f-852ea63e6f9c</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Elige el tipo «Mensual», tu programa y proyecto, y el mes y el año que rindes.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>En la pestaña «Listado de transacciones», presiona «Nuevo» por cada gasto.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Primero ingresa el comprobante de egreso (cómo pagaste) y adjúntalo escaneado. Después, el proveedor, el tipo de documento (boleta, factura…), su número, fecha y monto, el tipo de gasto (personal, operación o inversión), y adjunta los documentos que lo respaldan.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Presiona «Guardar y continuar» para seguir con el siguiente gasto, hasta cargar todos los del mes.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Presiona «Cerrar» y, en «Mis rendiciones», envíala al ministro de fe, que compara lo escaneado con los originales y la pasa al encargado ejecutor.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Quien tiene el rol de encargado ejecutor la revisa, presiona «Enviar para firma», la firma con su firma electrónica y, ya «Firmada», la envía al Ministerio con el ícono del avión.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Rendir el mes</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Hazlo dentro de los primeros 15 días hábiles del mes siguiente.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 (CGR); Res. 2/2026 CGR, art. 25 N°2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Rendir un mes sin movimiento</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Si ese mes no tuviste gastos, igual rindes: ve a «Mis rendiciones» y presiona «Nuevo».</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/4._Manual_Ejecutor_Rendicion_sin_Movimientos.pdf/89ce071f-508f-3f4b-885f-e796d8d3b5d7</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 04 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Rendir un mes sin movimiento</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Elige el tipo «Sin movimiento», tu programa y proyecto, y el mes y el año. Presiona «Guardar».</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 04 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Rendir un mes sin movimiento</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Revisa el formulario en borrador con la lupa y presiona «Cerrar».</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 04 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Rendir un mes sin movimiento</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Presiona «Enviar»: como no hay documentos que revisar, va directo al encargado ejecutor.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 04 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Rendir un mes sin movimiento</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Quien tiene el rol de encargado ejecutor la revisa, presiona «Enviar para firma», la firma con su firma electrónica y, ya «Firmada», la envía al Ministerio con el ícono del avión.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 04 (CGR); Rex 3391, punto 5.3.1 a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Corregir una rendición devuelta</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>En «Mis rendiciones», busca la que está «Observada» y abre su expediente.</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/7.Manual_Ejecutor_de+_Correccion_de_Rendicion_Devuelta_por_su_otorgante.pdf/56344e31-bb9c-ce57-5259-4798760b7732</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 07 (CGR); Rex 3391, punto 5.3.1 e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Corregir una rendición devuelta</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>En «Listado de transacciones», lee el comentario de cada gasto «Rendida observada».</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 07 (CGR); Rex 3391, punto 5.3.1 e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Corregir una rendición devuelta</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Corrige cada uno con el lápiz (sus datos o sus documentos) y presiona «Guardar»: queda «Rendida corregida».</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 07 (CGR); Rex 3391, punto 5.3.1 e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Corregir una rendición devuelta</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>El monto solo puede quedar igual o menor. Si el error está en el monto, o necesitas eliminar un gasto de una rendición que no es la última, pídelo en «Consulte aquí».</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 07 (CGR); Rex 3391, punto 5.3.1 e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Corregir una rendición devuelta</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Envíala de nuevo al ministro de fe: sigue el mismo camino que una rendición mensual.</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 07 (CGR); Rex 3391, punto 5.3.1 e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Corregir una rendición devuelta</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Hazlo dentro del plazo para corregir (mira «¿Qué hago si…?», «Me observaron un gasto o una actividad»).</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 07 (CGR); Rex 3391, punto 5.3.1 e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Cerrar el proyecto</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Puedes pedir el cierre cuando no te queden rendiciones en curso: menú «Proyectos» › «Solicitud cierre de proyectos».</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/11._Manual_Ejecutor_Cierre_de_Proyecto.pdf/2dc099f9-93d1-678d-d83b-ac943538acf6</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 11 (CGR); Rex 3391, punto 5.3.1 g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Cerrar el proyecto</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Busca tu proyecto, presiona el ícono para solicitar el cierre y confirma con «Sí».</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 11 (CGR); Rex 3391, punto 5.3.1 g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Cerrar el proyecto</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>En «Mis cierres proyecto», edita la solicitud y adjunta en «Documentación complementaria» el informe de término y, si devolviste dinero, el comprobante y la cartola del reintegro.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 11 (CGR); Rex 3391, punto 5.3.1 g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Cerrar el proyecto</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Envíala al ministro de fe; después el encargado ejecutor la firma y la envía al Ministerio con el ícono del avión.</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 11 (CGR); Rex 3391, punto 5.3.1 g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Cerrar el proyecto</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Si te quedó dinero sin gastar o te rechazaron gastos, devuélvelo antes: solo se cierran los proyectos sin saldo pendiente.</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 11 (CGR); Rex 3391, punto 5.3.1 g)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1703,7 +3396,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2474,7 +4167,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2882,7 +4575,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3190,7 +4883,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3448,7 +5141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8596,7 +10289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -8999,6 +10692,29 @@
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>0.4.0-prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>46318</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en el programa: «SISREC paso a paso», con 7 trámites explicados y el enlace a cada manual de la Contraloría, y «¿Qué hago si…?», con qué hacer, en qué plazo y quién firma en las situaciones más frecuentes.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Manuales SISREC del ejecutor (CGR); Rex 3096, Instr. 4.3, Sección 3.01</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>0.5.0-prueba</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reglas v11: programa 0.6.0-prueba con descarga y huella (actualización automática)
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
     </row>
     <row r="3">
@@ -500,7 +500,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.5.0-prueba</t>
+          <t>0.6.0-prueba</t>
         </is>
       </c>
     </row>
@@ -510,280 +510,308 @@
           <t>Descarga</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.6.0-prueba/Instalar-GuiaRendicion-0.6.0-prueba.exe</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Huella</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>DD66A22A321675EF9C678942E0BF49265085AE6327E6DADBF8004D2C56FB61DA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Contenido</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Reglas v2. Capa común: Rex 3092 a 3097, 3390 y 3391 de 2025 y Rex 1523 de 2024 (Subsecretaría de las Culturas y las Artes); Memos 02/1264, 02/566, 02/580, 02/064, 02/872, 02/978, 02/1283, 02/490, 02/306, 06/455 y 06/561; dictámenes de la CGR; Res. 30/2015 y Res. 2/2026 de Contraloría. Capa por fondo: bases de la Convocatoria 2027, tanda 1 (Fondart Regional y Libro), para convenios firmados desde el 01-01-2027.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="2" t="inlineStr"/>
-    </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Cómo editar</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>1. No cambies los nombres de las hojas ni de las columnas (fila 1): el programa los busca tal cual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>2. Una regla por fila.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>3. VigenteDesde y VigenteHasta: rango de fechas de firma del convenio en que aplica la regla (si no se conoce la firma, se usa la fecha de la resolución que lo aprueba; Memo 02/580). Vacío = sin límite.</t>
+          <t>2. Una regla por fila.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>4. Fondo y Linea: "Todos" y "Todas" para reglas comunes. Para un fondo o una línea, escribe su nombre o una parte, como aparece en la postulación (ej. Fondart Regional / Creación Artística): el programa busca esas palabras completas dentro del nombre.</t>
+          <t>3. VigenteDesde y VigenteHasta: rango de fechas de firma del convenio en que aplica la regla (si no se conoce la firma, se usa la fecha de la resolución que lo aprueba; Memo 02/580). Vacío = sin límite.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>5. TipoPersona: Todas, Natural o Juridica.</t>
+          <t>4. Fondo y Linea: "Todos" y "Todas" para reglas comunes. Para un fondo o una línea, escribe su nombre o una parte, como aparece en la postulación (ej. Fondart Regional / Creación Artística): el programa busca esas palabras completas dentro del nombre.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>6. PalabrasClave: en minúsculas y separadas por punto y coma; las tildes no importan.</t>
+          <t>5. TipoPersona: Todas, Natural o Juridica.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>7. Plazos: no cambies la columna Clave, la usa el programa. Puedes cambiar Cantidad, Unidad y los textos.</t>
+          <t>6. PalabrasClave: en minúsculas y separadas por punto y coma; las tildes no importan.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>6b. Las palabras clave se comparan por palabra completa (también en plural). Si un gasto calza con varios subítems, gana el de mayor Prioridad; a igual prioridad, el de la palabra clave más larga.</t>
+          <t>7. Plazos: no cambies la columna Clave, la usa el programa. Puedes cambiar Cantidad, Unidad y los textos.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>6c. ReglasGenerales.Seccion: Gastos, Proyecto, Entrega o Cofinanciamiento. Define en qué parte de la guía aparece la regla.</t>
+          <t>6b. Las palabras clave se comparan por palabra completa (también en plural). Si un gasto calza con varios subítems, gana el de mayor Prioridad; a igual prioridad, el de la palabra clave más larga.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>6d. En los textos puedes escribir [tu folio]: el programa lo reemplaza por el folio del proyecto.</t>
+          <t>6c. ReglasGenerales.Seccion: Gastos, Proyecto, Entrega o Cofinanciamiento. Define en qué parte de la guía aparece la regla.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>8. Al publicar una versión nueva, sube el número de Version.</t>
+          <t>6d. En los textos puedes escribir [tu folio]: el programa lo reemplaza por el folio del proyecto.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>9. Novedades: si la versión nueva cambia algo para los responsables, agrega en la hoja Novedades una fila por cambio, con el número de la versión nueva. El programa las muestra hasta que el responsable las marca como leídas. Si la novedad anuncia algo que solo trae un programa nuevo, escribe en DesdePrograma la versión que lo trae (ej. 0.3.1-prueba): los programas anteriores no la muestran. Vacío = la ven todos.</t>
+          <t>8. Al publicar una versión nueva, sube el número de Version.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>10. Programa y Descarga (filas de arriba): la última versión del programa (ej. 0.3.0) y el enlace https:// a su instalador. Si un programa instalado es más viejo, al abrirse avisa y muestra el enlace; si Descarga está vacía, pide el instalador al supervisor. Cámbialas solo cuando el instalador nuevo ya esté disponible en ese enlace.</t>
+          <t>9. Novedades: si la versión nueva cambia algo para los responsables, agrega en la hoja Novedades una fila por cambio, con el número de la versión nueva. El programa las muestra hasta que el responsable las marca como leídas. Si la novedad anuncia algo que solo trae un programa nuevo, escribe en DesdePrograma la versión que lo trae (ej. 0.3.1-prueba): los programas anteriores no la muestran. Vacío = la ven todos.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>11. Feriados: los feriados nacionales, para contar días hábiles (por ejemplo, el plazo de 15 días hábiles de cada rendición mensual). Agrega los del año siguiente antes de que empiece y los feriados por elecciones cuando se fijen. Los regionales no se cuentan (pregunta abierta a Jurídico).</t>
+          <t>10. Programa, Descarga y Huella (filas de arriba): la última versión del programa (ej. 0.6.0-prueba), el enlace https:// a su instalador (la release de guia-rendicion-reglas en GitHub) y la huella SHA-256 de ese instalador. Si un programa instalado es más viejo, al abrirse avisa; desde la 0.6.0, con la huella ofrece descargarlo, comprueba que la huella coincida e instala solo. Cámbialas solo cuando el instalador nuevo ya esté publicado en ese enlace, y calcula la huella del archivo publicado (PowerShell: Get-FileHash).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>12. Topes: el porcentaje máximo del monto pedido al fondo que puede sumar un subítem, según las bases de cada línea. El programa avisa si la postulación lo pasa.</t>
+          <t>11. Feriados: los feriados nacionales, para contar días hábiles (por ejemplo, el plazo de 15 días hábiles de cada rendición mensual). Agrega los del año siguiente antes de que empiece y los feriados por elecciones cuando se fijen. Los regionales no se cuentan (pregunta abierta a Jurídico).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>13. Glosario: términos que el programa explica en pantalla y en la guía.</t>
+          <t>12. Topes: el porcentaje máximo del monto pedido al fondo que puede sumar un subítem, según las bases de cada línea. El programa avisa si la postulación lo pasa.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>14. Etapas: los textos de «Así avanza tu proyecto» en la guía, uno por fila. Orden 1 a 7 son las etapas y 8 el desvío «¿Necesitas cambiar algo?»; no cambies esos números, porque el programa pone las fechas del responsable en las etapas 1, 2, 4 y 6 y en el desvío. Las filas con el mismo Orden llevan el mismo nombre en Etapa. Parte: Intro, Tú, Ministerio, Plazos u Ojo; dentro de cada etapa las partes salen en el orden de las filas. Lo que rige solo con la Res. 30/2015 lleva VigenteHasta 30-06-2026, y lo de la Res. 2/2026, VigenteDesde 01-07-2026.</t>
+          <t>13. Glosario: términos que el programa explica en pantalla y en la guía.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>15. Situaciones: «¿Qué hago si…?». Una fila por situación (o una por norma o tipo de persona, si cambia): qué hacer, el plazo y quién firma (estos dos pueden ir vacíos). Las filas con el mismo nombre se muestran juntas; en los textos puedes escribir [tu folio].</t>
+          <t>14. Etapas: los textos de «Así avanza tu proyecto» en la guía, uno por fila. Orden 1 a 7 son las etapas y 8 el desvío «¿Necesitas cambiar algo?»; no cambies esos números, porque el programa pone las fechas del responsable en las etapas 1, 2, 4 y 6 y en el desvío. Las filas con el mismo Orden llevan el mismo nombre en Etapa. Parte: Intro, Tú, Ministerio, Plazos u Ojo; dentro de cada etapa las partes salen en el orden de las filas. Lo que rige solo con la Res. 30/2015 lleva VigenteHasta 30-06-2026, y lo de la Res. 2/2026, VigenteDesde 01-07-2026.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="2" t="inlineStr">
         <is>
+          <t>15. Situaciones: «¿Qué hago si…?». Una fila por situación (o una por norma o tipo de persona, si cambia): qué hacer, el plazo y quién firma (estos dos pueden ir vacíos). Las filas con el mismo nombre se muestran juntas; en los textos puedes escribir [tu folio].</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
           <t>16. SISREC: un paso por fila, numerados desde 1 en cada trámite. En la fila del paso 1 va el enlace https:// al manual de la Contraloría.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="2" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Pendiente de validar</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Cambios en la versión 10</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
-        </is>
-      </c>
-    </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cambios en la versión 9</t>
+          <t>Cambios en la versión 11</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
+          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cambios en la versión 8</t>
+          <t>Cambios en la versión 10</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
+          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Cambios en la versión 4</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -10289,7 +10317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10715,6 +10743,25 @@
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>0.5.0-prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en el programa: cuando sale una versión nueva, te ofrece descargarla e instalarla sola (tu proyecto se mantiene), y el botón «Créditos» muestra quién desarrolló el programa y con qué herramientas.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>0.6.0-prueba</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reglas v12: prórroga sin fecha de vencimiento, aceptación en SISREC y programa 0.6.1-prueba
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -479,7 +479,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2">
@@ -500,7 +500,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.6.0-prueba</t>
+          <t>0.6.1-prueba</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.6.0-prueba/Instalar-GuiaRendicion-0.6.0-prueba.exe</t>
+          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.6.1-prueba/Instalar-GuiaRendicion-0.6.1-prueba.exe</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>DD66A22A321675EF9C678942E0BF49265085AE6327E6DADBF8004D2C56FB61DA</t>
+          <t>046033552C573137FB95F1AB73773E8DF65BBF7E99FE434032B190DC9E347901</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes.</t>
+          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes. (i) prórroga: la Rex 3096 pide 30 días corridos antes de que venza el convenio, pero el convenio 2026 revisado rige «hasta la ejecución total del proyecto» (sin fecha de vencimiento) y acepta la prórroga hasta antes del término de la ejecución: el programa recomienda pedirla 30 días antes del término.</t>
         </is>
       </c>
     </row>
@@ -700,118 +700,130 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cambios en la versión 11</t>
+          <t>Cambios en la versión 12</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
+          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cambios en la versión 10</t>
+          <t>Cambios en la versión 11</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
+          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 9</t>
+          <t>Cambios en la versión 10</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
+          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cambios en la versión 8</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 4</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -908,7 +920,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Al menos 30 días corridos antes de que venza tu convenio. Se aceptan hasta 2 prórrogas, y el plazo total puede crecer como máximo la mitad de lo que dura tu proyecto. Si tu garantía es una letra de cambio, entrega la nueva dentro de 2 días desde que te notifican la aprobación.</t>
+          <t>Al menos 30 días corridos antes de que venza tu convenio (si no tiene fecha de vencimiento, antes de que termine la ejecución). Se aceptan hasta 2 prórrogas, y el plazo total puede crecer como máximo la mitad de lo que dura tu proyecto. Si tu garantía es una letra de cambio, entrega la nueva dentro de 2 días desde que te notifican la aprobación.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2581,12 +2593,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Pide la prórroga al menos 30 días corridos antes de que venza el convenio.</t>
+          <t>Pide la prórroga al menos 30 días corridos antes de que venza tu convenio. Y si tu convenio no tiene fecha de vencimiento (por ejemplo, si dice que rige hasta la ejecución total del proyecto), cuéntalos desde el término de la ejecución: tu convenio la acepta hasta antes de ese término, pero no esperes al último día.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Rex 3096, Instr. 4.3, Glosario (Prórroga)</t>
+          <t>Rex 3096, Instr. 4.3, Glosario (Prórroga); tu convenio (cláusula de prórroga)</t>
         </is>
       </c>
       <c r="G2" s="5" t="n"/>
@@ -4812,7 +4824,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Una extensión del plazo de ejecución del proyecto. Se pide antes de que venza el convenio, con al menos 30 días corridos de anticipación.</t>
+          <t>Una extensión del plazo de ejecución del proyecto. Se pide con al menos 30 días corridos de anticipación al vencimiento del convenio o, si el convenio no tiene fecha de vencimiento, al término de la ejecución.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -10317,7 +10329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10762,6 +10774,29 @@
       <c r="E22" s="2" t="inlineStr">
         <is>
           <t>0.6.0-prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>46319</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en «Mi proyecto»: anota cuándo aceptaste la transferencia en SISREC y tus rendiciones mensuales se cuentan desde ese mes. Además, tu calendario trae la fecha recomendada para pedir una prórroga aunque tu convenio no tenga fecha de vencimiento, y las renovaciones de tu garantía hasta el cierre del convenio.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3391, punto 5.3.1; Rex 3096, Instr. 4.3, Glosario (Prórroga); Memo 02/1264</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>0.6.1-prueba</t>
         </is>
       </c>
     </row>
@@ -26288,7 +26323,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Prórroga (más plazo para tu proyecto): pídela al menos 30 días corridos antes de que venza tu convenio, con un nuevo cronograma y un informe de lo que llevas hecho. Se aceptan hasta 2 prórrogas, y el plazo total puede crecer como máximo la mitad de lo que dura tu proyecto. Si te la aprueban, renueva tu garantía para que cubra el nuevo plazo.</t>
+          <t>Prórroga (más plazo para tu proyecto): pídela al menos 30 días corridos antes de que venza tu convenio (o antes de que termine la ejecución, si tu convenio no tiene fecha de vencimiento), con un nuevo cronograma y un informe de lo que llevas hecho. Se aceptan hasta 2 prórrogas, y el plazo total puede crecer como máximo la mitad de lo que dura tu proyecto. Si te la aprueban, renueva tu garantía para que cubra el nuevo plazo.</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Reglas v13 firmadas: hojas Retenciones y Fuentes; programa 0.7.0-prueba con descarga y huella
Desde la 0.7.0 el programa acepta las reglas solo con reglas.xlsx.firma.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -24,6 +24,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glosario" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ErroresFrecuentes" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReglasBases" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retenciones" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Subitems'!$A$1:$F$29</definedName>
@@ -46,7 +48,7 @@
     <numFmt numFmtId="164" formatCode="dd-mm-yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,8 +59,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +74,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,6 +111,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -465,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -479,7 +491,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2">
@@ -489,7 +501,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="3">
@@ -500,7 +512,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.6.1-prueba</t>
+          <t>0.7.0-prueba</t>
         </is>
       </c>
     </row>
@@ -512,7 +524,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.6.1-prueba/Instalar-GuiaRendicion-0.6.1-prueba.exe</t>
+          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.7.0-prueba/Instalar-GuiaRendicion-0.7.0-prueba.exe</t>
         </is>
       </c>
     </row>
@@ -524,7 +536,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>046033552C573137FB95F1AB73773E8DF65BBF7E99FE434032B190DC9E347901</t>
+          <t>A75CB6B2909528080B201764CFCC67DB35A80BE0E2E69E84006B94F51AF7CA7B</t>
         </is>
       </c>
     </row>
@@ -682,148 +694,173 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>17. Retenciones: la retención de las boletas de honorarios de cada año (Anio y Porcentaje del monto bruto, como 15,25). El programa la muestra en los gastos de honorarios y revisa con ella las boletas que adjunta el responsable. Agrega el año siguiente antes de que empiece.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Pendiente de validar</t>
-        </is>
-      </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes. (i) prórroga: la Rex 3096 pide 30 días corridos antes de que venza el convenio, pero el convenio 2026 revisado rige «hasta la ejecución total del proyecto» (sin fecha de vencimiento) y acepta la prórroga hasta antes del término de la ejecución: el programa recomienda pedirla 30 días antes del término.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
+          <t>18. Fuentes: las normas y documentos de la Biblioteca, uno por fila, con el enlace a su publicación oficial (https://). Sale del inventario de Documentación; nunca agregues documentos con datos personales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr"/>
+    </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Cambios en la versión 12</t>
+          <t>Pendiente de validar</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Cambios en la versión 11</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
+          <t>Contradicciones abiertas (detalle en la matriz de plazos, preguntas P1 a P13, y en el borrador de bases 2027, C1 a C7): (a) los instructivos y la Rex 3391 citan la Res. 30/2015, derogada desde el 01-07-2026; (b) plazos de la Res. 2/2026: el programa usa la interpretación de la matriz mientras Jurídico no responda; (c) firma electrónica vs. «solo originales»; (d) cofinanciamiento voluntario: ¿se rinde?; (e) medicamentos: permitidos en manutención y prohibidos como no financiables; (f) combustible y peajes sin regla; (g) la Rex 3391 pide más respaldos que la Rex 3096 (factura en vez de boleta): se suman y se pide factura «si puedes»; (h) finiquitos e indemnizaciones: Rex 3096, Rex 3391 y la guía de contratación 2027 no coinciden: se pide consultar antes. (i) prórroga: la Rex 3096 pide 30 días corridos antes de que venza el convenio, pero el convenio 2026 revisado rige «hasta la ejecución total del proyecto» (sin fecha de vencimiento) y acepta la prórroga hasta antes del término de la ejecución: el programa recomienda pedirla 30 días antes del término.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 10</t>
+          <t>Cambios en la versión 13</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
+          <t>Hojas Retenciones (honorarios 2026 a 2028) y Fuentes (87 normas y documentos con su enlace oficial). Una novedad para el programa 0.7.0-prueba: presupuesto, revisión de documentos, carpeta para SISREC, informe IN17, avisos y Biblioteca.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cambios en la versión 9</t>
+          <t>Cambios en la versión 12</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
+          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cambios en la versión 8</t>
+          <t>Cambios en la versión 11</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
+          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 10</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>Cambios en la versión 5</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 4</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -10323,13 +10360,2044 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Anio</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Porcentaje</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Guía para una correcta contratación, Concurso General 2027, punto 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Guía para una correcta contratación, Concurso General 2027, punto 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>2028</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Guía para una correcta contratación, Concurso General 2027, punto 9</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D88"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Documento</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>Enlace</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Res N° 30 de fecha 28-03-2015 - Normas de rendición de cuentas, régimen anterior (CGR)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CGR: normas de rendición de cuentas (régimen de convenios anteriores al 01-07-2026)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1075796</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 1858 de fecha 23-09-2023 - Uso obligatorio del SISREC (CGR)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CGR: uso obligatorio del SISREC</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1196159</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Instructivo N° IN17 de fecha 11-05-2026 - Formato del informe de ejecución de actividades (CGR)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CGR: formato obligatorio del informe de ejecución de actividades (Res. 2/2026)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.investchile.gob.cl/wp-content/uploads/2026/08/Instructivo-N%C2%B0-IN17-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 1523 de fecha 28-06-2024 - Prórrogas en modalidad simplificada</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>MINCAP: modalidad simplificada de prórrogas</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Manual e instructivos del Ministerio</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1204555</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 6 de fecha 03-06-2021 - Reglamento del Fondart</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Reglamento del FONDART</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1160647</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 587 de fecha 27-09-1993 - Reglamento del Fondo del Libro</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Reglamento del Fondo del Libro y la Lectura</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=14452</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 187 de fecha 25-10-2004 - Reglamento del Fondo de la Música</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Reglamento del Fondo de la Música</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=231661</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 151 de fecha 12-09-2005 - Reglamento del Fondo Audiovisual</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Reglamento del Fondo Audiovisual (texto sustituido por DTO 176/2011)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=241853</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 9 de fecha 03-06-2021 - Reglamento de Artes Escénicas</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Reglamento de la Ley 21.175 (Artes Escénicas)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1160648</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 19.862 de fecha 08-02-2003 - Registro de receptores de fondos públicos</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Registro de receptores de fondos públicos</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=207438</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 19.799 de fecha 12-04-2002 - Documentos y firma electrónica</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Documentos y firma electrónica</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=196640</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 21.722 de fecha 13-12-2024 - Presupuestos 2025</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Ley de Presupuestos 2025 (declaración jurada)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1209325</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 21.796 de fecha 12-12-2025 - Presupuestos 2026</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Ley de Presupuestos 2026</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1219410</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Oficio Circular N° 11 de fecha 13-06-2024 - Transferencias a instituciones privadas (Hacienda)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Hacienda: convenios de transferencias a instituciones privadas</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dipres.gob.cl/598/articles-335411_doc_pdf.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 21.389 de fecha 18-11-2021 - Registro de deudores de pensiones de alimentos</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Registro de deudores de pensiones de alimentos (retención)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1168463</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>DFL N° 1 de fecha 16-01-2003 - Código del Trabajo</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Código del Trabajo (menores de edad, trabajadores de artes y espectáculos)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Normas tributarias y laborales</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=207436</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 18.985 de fecha 28-06-1990 - Donaciones culturales</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Ley de Donaciones Culturales (art. 8)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=30353</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>DL N° 824 de fecha 31-12-1974 - Impuesto a la Renta</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Ley sobre Impuesto a la Renta (sueldo empresarial, honorarios)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Normas tributarias y laborales</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=6368</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>DL N° 825 de fecha 31-12-1974 - Impuesto al Valor Agregado (IVA)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Ley del IVA</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Normas tributarias y laborales</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=6369</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>DL N° 830 de fecha 31-12-1974 - Código Tributario</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Código Tributario</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Normas tributarias y laborales</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=6374</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 45 de fecha 01-09-2003 - Documentos tributarios electrónicos (SII)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>SII: documentos tributarios electrónicos (página web)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Normas tributarias y laborales</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sii.cl/documentos/resoluciones/2003/reso45.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>DL N° 1.263 de fecha 28-11-1975 - Administración Financiera del Estado</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Administración Financiera del Estado (arts. 54 y 55)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=6536</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 10.336 de fecha 10-07-1964 - Organización de la Contraloría, texto refundido</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Organización y atribuciones de la Contraloría (texto de la CGR)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/documents/451102/1887680/PDF+Ley+10336/d6559f9f-c3b4-4b33-ab15-3e41904a25e7</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 19.880 de fecha 29-05-2003 - Procedimientos administrativos</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Procedimientos administrativos (plazos en días hábiles)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=210676</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>DFL N° 1-19.653 de fecha 17-11-2001 - Bases Generales de la Administración del Estado</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Bases Generales de la Administración del Estado</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=191865</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 854 de fecha 02-12-2004 - Clasificador presupuestario</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Clasificador presupuestario (subtítulos 24 y 33)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=233184</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Res N° 10 de fecha 30-06-2021 - Normas de auditoría (CGR)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>CGR: normas de auditoría</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1162083</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Res N° 36 de fecha 23-12-2024 - Exención de toma de razón (CGR)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>CGR: exención de toma de razón</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1209651</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 1962 de fecha 04-10-2022 - Normas de control interno (CGR)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>CGR: normas de control interno</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.portaltransparencia.cl/PortalPdT/documents/10179/62801/Res.+Exenta+NA%CC%82%201.962+de+2022.+Aprueba+normas+sobre+control+interno+de+la+ContralorA%CC%83-a+General+de+la+RepA%CC%83%C2%BAblica.pdf/eda50647-cfd7-499d-8987-6774920e0d74</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 181 de fecha 17-08-2002 - Reglamento de firma electrónica</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Reglamento de la Ley 19.799</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=201668</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 21.640 de fecha 18-12-2023 - Presupuestos 2024</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Ley de Presupuestos 2024 (base del Oficio Circular 11)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1199318</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 17.336 de fecha 02-10-1970 - Propiedad intelectual</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Propiedad intelectual</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=28933</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 19.733 de fecha 04-06-2001 - Libertad de opinión y depósito legal</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Libertad de opinión (art. 14, depósito legal)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Leyes y reglamentos de los Fondos</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=186049</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 21.210 de fecha 24-02-2020 - Modernización tributaria</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Modernización tributaria</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Normas tributarias y laborales</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1142667</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 141 de fecha 30-12-2021 - Cambio de sujeto del IVA (SII)</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>SII: cambio de sujeto del IVA (relevancia dudosa)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Normas tributarias y laborales</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.sii.cl/normativa_legislacion/resoluciones/2021/reso141.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2211 de fecha 17-11-2016 - Manual anterior de control de proyectos (CNCA)</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>CNCA: manual anterior de control y supervisión de proyectos de los Fondos de Cultura (derogado por la Rex 3092)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Normas anteriores del CNCA</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>https://transparenciaactiva.cultura.gob.cl/uploads/marcoNormativo/1527928c312a5bd169fbb83dd8c35c8631cbbff1.PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Manual de Normas Gráficas MINCAP, versión 2023</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>MINCAP: manual de normas gráficas, versión 2023 (uso del logo del Ministerio)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Manual e instructivos del Ministerio</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cultura.gob.cl/wp-content/uploads/2023/04/normas-graficas-mincap-2023.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 1339 de fecha 11-08-2023 - Consulta del registro de deudores de alimentos</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Subsecretaría: procedimiento interno de consulta del Registro Nacional de Deudores de Alimentos (art. 36 de la Ley 21.389)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Manual e instructivos del Ministerio</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1195013</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2398 de fecha 23-12-2015 - Castigo de créditos incobrables (CNCA)</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>CNCA: procedimiento para el castigo de créditos declarados incobrables (deudas de beneficiarios que el Consejo de Defensa del Estado declara incobrables)</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Normas anteriores del CNCA</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>https://transparenciaactiva.cultura.gob.cl/uploads/marcoNormativo/6289f60e16fc504c41b4dcee3532d417e81a7c44.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 1444 de fecha 12-04-2013 - Protocolo de colaboración con el CDE (CNCA)</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>CNCA: protocolo de procedimiento y colaboración con el Consejo de Defensa del Estado (cobro judicial a beneficiarios)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Normas anteriores del CNCA</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>https://transparenciaactiva.cultura.gob.cl/uploads/marcoNormativo/f4e898193e80428367076e49448dd578ef0ea487.PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° E324651 de fecha 22-03-2023 - Instrucciones sobre cuentas corrientes bancarias (CGR)</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>CGR: instrucciones sobre manejo y control de cuentas corrientes bancarias</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/E324651N23/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 50.611 de fecha 11-09-2009 - Gastos de habilitación de oficina con recursos transferidos (CGR)</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>CGR: no procede imputar gastos de habilitación de oficina a recursos transferidos</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/050611N09/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 6.135 de fecha 31-01-2012 - Gastos de personas jurídicas sin fines de lucro con fondos públicos (CGR)</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>CGR: gastos de personas jurídicas sin fines de lucro con fondos estatales</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/006135N12/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 14.853 de fecha 26-04-2017 - Gastos administrativos y operacionales en transferencias (CGR)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>CGR: concepto de gastos administrativos y operacionales en transferencias</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/014853N17/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Decreto N° 110 de fecha 20-03-1979 - Reglamento de personalidad jurídica de corporaciones y fundaciones</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Reglamento sobre concesión de personalidad jurídica a corporaciones y fundaciones</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Administración y finanzas públicas</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=135904</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 01 - Administrador del SISREC (CGR)</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Administrador del SISREC</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/1._Manual_de_Administrador_del_SISREC_Ejecutor.pdf/38415c08-57d3-5dcc-1c96-e48297fd1cee</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 02 - Ingreso de un proveedor (CGR)</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Ingreso de un proveedor</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/2._Manual_Ejecutor_Ingreso_de_un_Proveedor.pdf/e6fc195a-c703-91a8-e5ed-b7ae3229aa1a</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 03 - Aceptación o rechazo de transferencia (CGR)</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Aceptación o rechazo de transferencia</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/3._Manual_Ejecutor_Aceptacion_o_rechazo_de_Transferencia.pdf/69905a76-8959-bfe3-7768-b3c824077ba1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 04 - Rendición sin movimientos (CGR)</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Rendición sin movimientos</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/4._Manual_Ejecutor_Rendicion_sin_Movimientos.pdf/89ce071f-508f-3f4b-885f-e796d8d3b5d7</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 05 - Rendición mensual (CGR)</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Rendición mensual</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/5._Manual_Ejecutor_Rendicion_Mensual.pdf/003c9e08-83a5-07c4-618f-852ea63e6f9c</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 07 - Corrección de rendición devuelta (CGR)</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Corrección de rendición devuelta</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/7.Manual_Ejecutor_de+_Correccion_de_Rendicion_Devuelta_por_su_otorgante.pdf/56344e31-bb9c-ce57-5259-4798760b7732</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 08 - Revisión del ministro de fe (CGR)</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Revisión del ministro de fe</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/8._Manual_Ejecutor_Revision_Ministro_de_Fe.pdf/00c9a767-fe20-b0b8-ed35-496da41dd47e</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 09 - Carga masiva en rendición mensual (CGR)</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Carga masiva en rendición mensual</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/9._Manual_Ejecutor_Carga_Masiva_en_Rendicion_Mensual.docx/f7f742bc-80b4-bbf5-a9d5-74b4f4372dcd</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 10 - Perfil de lectura (CGR)</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Perfil de lectura</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/10._Manual_Ejecutor_Perfil_Lectura.pdf/1843f44c-ee8a-2a46-c314-5e8575aee31a</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Ejecutor 11 - Cierre de proyecto (CGR)</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Cierre de proyecto</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80411/11._Manual_Ejecutor_Cierre_de_Proyecto.pdf/2dc099f9-93d1-678d-d83b-ac943538acf6</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Otorgante 12 - Aprobación de rendición sin movimiento (CGR)</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Aprobación de rendición sin movimiento</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80413/12._Manual_Otorgante_Aprobacion_Rendicion_Sin_Movimiento.pdf/f12368bd-7a44-76e4-22e5-57d00e5fc588</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Otorgante 13 - Aprobación total de rendición mensual (CGR)</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Aprobación total de rendición mensual</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80413/13._Manual_Otorgante_Aprobacion_Total_Rendicion_Mensual.pdf/d41775ac-4197-6331-0006-3419ae0af289</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Otorgante 18 - Devolución de rendición (CGR)</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Devolución de rendición</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80413/18._Manual_Otorgante_Devolucion_Rendicion.pdf/3b2ef369-6c03-4a4e-2337-c99af4d8bd69</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Manual SISREC Otorgante 19 - Cierre de proyecto (CGR)</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Cierre de proyecto</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80413/19._Manual_Otorgante_Cierre_de_Proyecto.pdf/55170146-bc60-b99a-1bb1-30410847c2e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Preguntas frecuentes SISREC (CGR)</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Preguntas frecuentes SISREC</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/preguntas-frecuentes</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Glosario SISREC (CGR)</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Glosario SISREC</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>SISREC - Manuales de la Contraloría</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/75311/80415/glosario-sisrec.pdf/34021ab3-6895-9a50-aa38-e0234a545c87</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Formato tipo del informe de ejecución de actividades (CGR)</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Formato tipo del informe de ejecución de actividades</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Rendición de cuentas - Contraloría</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rendicioncuentas.cl/documents/d/guest/formato-tipo-informe-de-ejecucion-de-actividades</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Ley N° 20.880 de fecha 05-01-2016 - Probidad en la función pública</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Probidad en la función pública y prevención de conflictos de intereses</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcn.cl/leychile/navegar?idNorma=1086062</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 73.040 de fecha 31-12-2009 - Probidad administrativa (CGR)</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Probidad administrativa</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/073040N09/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 22.527 de fecha 30-04-2010 - Probidad de consejeros de CONADI (CGR)</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Probidad de consejeros de CONADI</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/022527N10/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 39.453 de fecha 15-07-2010 - Conflicto de intereses y probidad (CGR)</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Conflicto de intereses y probidad</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/039453N10/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 21.414 de fecha 25-03-2014 - Conflicto de interés de funcionario accionista (CGR)</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Conflicto de interés de funcionario accionista</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/021414N14/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° 17.083 de fecha 25-06-2019 - Funcionarios de CORFO pueden postular a sus fondos (CGR)</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Funcionarios de CORFO pueden postular a sus fondos</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/017083N19/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° E127439 de fecha 06-08-2021 - Donaciones privadas a municipios (CGR)</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Donaciones privadas a municipios</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/E127439N21/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Dictamen N° E174848 de fecha 15-10-2025 - Vigencia de jurisprudencia (CGR)</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>CGR: Vigencia de jurisprudencia</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Probidad</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.contraloria.cl/pdfbuscador/dictamenes/E174848N25/pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027 - Libro, Fomento a la Creación (aprobadas por Rex N° 2150)</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Bases del concurso: Libro y la Lectura · Fomento a la Creación</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/07/creacion-libro-2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2150 de fecha 27-07-2026 - Aprueba bases 2027 Libro, Fomento a la Creación</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Resolución que aprueba las bases: Libro y la Lectura · Fomento a la Creación</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/07/rex-2150-creacion-libro-2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2573 de fecha 01-09-2026 - Amplía plazo de postulación Libro, Fomento a la Creación</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Amplía el plazo de postulación: Libro y la Lectura · Fomento a la Creación</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/07/Rex-2573-ano-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027 - Libro, Fomento de la Lectura (aprobadas por Rex N° 2165)</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Bases del concurso: Libro y la Lectura · Fomento de la Lectura, Escritura y Comunicación Oral</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/07/fomento-lectura-libro-2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2165 de fecha 28-07-2026 - Aprueba bases 2027 Libro, Fomento de la Lectura</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Resolución que aprueba las bases: Libro y la Lectura · Fomento de la Lectura, Escritura y Comunicación Oral</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/07/rex-2165-fomento-lectura-libro-2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027 - Fondart Regional, Actividades Formativas (aprobadas por Rex N° 2261)</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Bases del concurso: Fondart Regional · Actividades Formativas</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/ActividadesFormativas-Regional2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2261 de fecha 05-08-2026 - Aprueba bases 2027 Fondart Regional, Actividades Formativas</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Resolución que aprueba las bases: Fondart Regional · Actividades Formativas</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/REX2261-ActividadesFormativas-Regional27.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027 - Fondart Regional, Culturas Regionales (aprobadas por Rex N° 2258)</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Bases del concurso: Fondart Regional · Culturas Regionales</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/CulturasRegionales-Regional2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2258 de fecha 05-08-2026 - Aprueba bases 2027 Fondart Regional, Culturas Regionales</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Resolución que aprueba las bases: Fondart Regional · Culturas Regionales</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/REX2258-CulturasReg-Regional27.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027 - Fondart Regional, Creación Artística (aprobadas por Rex N° 2262)</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Bases del concurso: Fondart Regional · Creación Artística, Innovación y Nuevos Formatos Creativos</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/CreacionArtistica-Regional2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2262 de fecha 05-08-2026 - Aprueba bases 2027 Fondart Regional, Creación Artística</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Resolución que aprueba las bases: Fondart Regional · Creación Artística, Innovación y Nuevos Formatos Creativos</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/REX2262-CreacionArt-Regional27.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027 - Fondart Regional, Difusión (aprobadas por Rex N° 2259)</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Bases del concurso: Fondart Regional · Difusión</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/Difusion-Regional2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2259 de fecha 05-08-2026 - Aprueba bases 2027 Fondart Regional, Difusión</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Resolución que aprueba las bases: Fondart Regional · Difusión</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/REX2259-DifusionReg-Regional27.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027 - Fondart Regional, Culturas Tradicionales (aprobadas por Rex N° 2260)</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Bases del concurso: Fondart Regional · Culturas Tradicionales</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/CulturasTradicionales-Regional2027.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2260 de fecha 05-08-2026 - Aprueba bases 2027 Fondart Regional, Culturas Tradicionales</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Resolución que aprueba las bases: Fondart Regional · Culturas Tradicionales</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/REX2260-CulturasTrad-Regional27.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Guía Concurso General 2027 - Correcta contratación</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Guía para una correcta contratación: Común · Todas las líneas del Concurso General 2027</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/08/guia-contrataciones.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Rex N° 2596 de fecha 02-09-2026 - Amplía plazo de postulación Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Amplía el plazo de postulación: Común · Varias líneas de la Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Bases Convocatoria 2027</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fondosdecultura.cl/wp-content/uploads/2026/09/Rex-2596-ano-2026.pdf</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -10797,6 +12865,29 @@
       <c r="E23" s="2" t="inlineStr">
         <is>
           <t>0.6.1-prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>46320</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo en el programa: anota lo que gastas y mira tu presupuesto; adjunta tus boletas, facturas y verificadores para que el programa los revise; arma la carpeta de cada mes para SISREC; llena el informe de actividades (formato IN17 de la Contraloría); recibe avisos de tus fechas al encender el computador; y busca las normas, con su enlace oficial, en la Biblioteca.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096; Instructivo IN17 (CGR); Guía para una correcta contratación, Concurso General 2027, punto 9</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>0.7.0-prueba</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reglas v14 firmadas: textos de la hoja Leeme y programa 0.7.1-prueba con descarga y huella
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2">
@@ -512,7 +512,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.7.0-prueba</t>
+          <t>0.7.1-prueba</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.7.0-prueba/Instalar-GuiaRendicion-0.7.0-prueba.exe</t>
+          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.7.1-prueba/Instalar-GuiaRendicion-0.7.1-prueba.exe</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>A75CB6B2909528080B201764CFCC67DB35A80BE0E2E69E84006B94F51AF7CA7B</t>
+          <t>639C374DA247FA0E9BA73B2EBC0A40D4AC3F3AB3FC6E85BCFFE43D7FCC73D518</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Reglas v2. Capa común: Rex 3092 a 3097, 3390 y 3391 de 2025 y Rex 1523 de 2024 (Subsecretaría de las Culturas y las Artes); Memos 02/1264, 02/566, 02/580, 02/064, 02/872, 02/978, 02/1283, 02/490, 02/306, 06/455 y 06/561; dictámenes de la CGR; Res. 30/2015 y Res. 2/2026 de Contraloría. Capa por fondo: bases de la Convocatoria 2027, tanda 1 (Fondart Regional y Libro), para convenios firmados desde el 01-01-2027.</t>
+          <t>Las reglas salen de estas normas (lo que cambió en cada versión está abajo, en «Cambios en la versión…»). Capa común: Rex 3092 a 3097, 3390 y 3391 de 2025 y Rex 1523 de 2024 (Subsecretaría de las Culturas y las Artes); Memos 02/1264, 02/566, 02/580, 02/064, 02/872, 02/978, 02/1283, 02/490, 02/306, 06/455 y 06/561; dictámenes de la CGR; Res. 30/2015 y Res. 2/2026 de Contraloría. Capa por fondo: bases de la Convocatoria 2027, tanda 1 (Fondart Regional y Libro), para convenios firmados desde el 01-01-2027. Las normas, con su enlace oficial, están en la hoja Fuentes.</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>8. Al publicar una versión nueva, sube el número de Version.</t>
+          <t>8. Al publicar una versión nueva, sube el número de Version. Después fírmala en el Mantenedor de reglas (pestaña «Firmar y publicar» → «Validar y firmar el Excel de reglas»), que deja reglas.xlsx.firma al lado del Excel, y sube los dos archivos juntos a guia-rendicion-reglas. Desde el programa 0.7.0, las reglas sin una firma válida se rechazan: si cambias el Excel después de firmarlo, aunque sea un texto, vuelve a firmarlo.</t>
         </is>
       </c>
     </row>
@@ -703,12 +703,16 @@
     <row r="28">
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>18. Fuentes: las normas y documentos de la Biblioteca, uno por fila, con el enlace a su publicación oficial (https://). Sale del inventario de Documentación; nunca agregues documentos con datos personales.</t>
+          <t>18. Fuentes: las normas y documentos de la Biblioteca, uno por fila, con el enlace a su publicación oficial (https://). Salen del inventario de Documentación; el Mantenedor agrega uno cuando aplicas el borrador de un documento que trae su enlace oficial. Nunca agregues documentos con datos personales (carpeta 13) ni de recursos humanos (carpeta 10).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>19. Canal de prueba: para probar una versión antes de publicarla para todos, súbela con su firma a la carpeta beta/ de guia-rendicion-reglas. Solo la bajan los computadores que se cambiaron con «GuiaRendicion.exe --canal beta» (vuelven con «--canal estable»); si beta/ está vacía, usan las de todos.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -722,145 +726,158 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 13</t>
+          <t>Cambios en la versión 14</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Hojas Retenciones (honorarios 2026 a 2028) y Fuentes (87 normas y documentos con su enlace oficial). Una novedad para el programa 0.7.0-prueba: presupuesto, revisión de documentos, carpeta para SISREC, informe IN17, avisos y Biblioteca.</t>
+          <t>Textos de esta hoja: la firma al publicar (paso 8), de dónde salen las Fuentes (paso 18), el canal de prueba (paso 19) y la fila Contenido. Programa 0.7.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella), y una novedad para ese programa: adjuntos, montos y copias del proyecto.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cambios en la versión 12</t>
+          <t>Cambios en la versión 13</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
+          <t>Hojas Retenciones (honorarios 2026 a 2028) y Fuentes (87 normas y documentos con su enlace oficial). Una novedad para el programa 0.7.0-prueba: presupuesto, revisión de documentos, carpeta para SISREC, informe IN17, avisos y Biblioteca.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cambios en la versión 11</t>
+          <t>Cambios en la versión 12</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
+          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cambios en la versión 10</t>
+          <t>Cambios en la versión 11</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
+          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cambios en la versión 9</t>
+          <t>Cambios en la versión 10</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
+          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cambios en la versión 8</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 4</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -12397,7 +12414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -12888,6 +12905,29 @@
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>0.7.0-prueba</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Mejoras en el programa: al adjuntar una boleta o factura, su total se suma a lo que gastaste ese mes, y el documento queda «lo tengo» solo si la revisión automática no encontró nada que revisar. «Guardar una copia…» guarda también tus archivos adjuntos, y si abres tu proyecto desde otra carpeta (un pendrive o la versión web), el programa lo trae a su carpeta con sus adjuntos.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Rex 3096, Instr. 4.2</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>0.7.1-prueba</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reglas v15 firmadas: la novedad de la v14 ya no menciona la versión web
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B44"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2">
@@ -730,154 +730,166 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 14</t>
+          <t>Cambios en la versión 15</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Textos de esta hoja: la firma al publicar (paso 8), de dónde salen las Fuentes (paso 18), el canal de prueba (paso 19) y la fila Contenido. Programa 0.7.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella), y una novedad para ese programa: adjuntos, montos y copias del proyecto.</t>
+          <t>La novedad de la versión 14 ya no menciona la versión web, que se descartó el 26-10-2026: el programa es solo para Windows. Ninguna regla cambia.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cambios en la versión 13</t>
+          <t>Cambios en la versión 14</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Hojas Retenciones (honorarios 2026 a 2028) y Fuentes (87 normas y documentos con su enlace oficial). Una novedad para el programa 0.7.0-prueba: presupuesto, revisión de documentos, carpeta para SISREC, informe IN17, avisos y Biblioteca.</t>
+          <t>Textos de esta hoja: la firma al publicar (paso 8), de dónde salen las Fuentes (paso 18), el canal de prueba (paso 19) y la fila Contenido. Programa 0.7.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella), y una novedad para ese programa: adjuntos, montos y copias del proyecto.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cambios en la versión 12</t>
+          <t>Cambios en la versión 13</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
+          <t>Hojas Retenciones (honorarios 2026 a 2028) y Fuentes (87 normas y documentos con su enlace oficial). Una novedad para el programa 0.7.0-prueba: presupuesto, revisión de documentos, carpeta para SISREC, informe IN17, avisos y Biblioteca.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cambios en la versión 11</t>
+          <t>Cambios en la versión 12</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
+          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cambios en la versión 10</t>
+          <t>Cambios en la versión 11</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
+          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cambios en la versión 9</t>
+          <t>Cambios en la versión 10</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
+          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cambios en la versión 8</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 4</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>
@@ -12917,7 +12929,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Mejoras en el programa: al adjuntar una boleta o factura, su total se suma a lo que gastaste ese mes, y el documento queda «lo tengo» solo si la revisión automática no encontró nada que revisar. «Guardar una copia…» guarda también tus archivos adjuntos, y si abres tu proyecto desde otra carpeta (un pendrive o la versión web), el programa lo trae a su carpeta con sus adjuntos.</t>
+          <t>Mejoras en el programa: al adjuntar una boleta o factura, su total se suma a lo que gastaste ese mes, y el documento queda «lo tengo» solo si la revisión automática no encontró nada que revisar. «Guardar una copia…» guarda también tus archivos adjuntos, y si abres tu proyecto desde otra carpeta (por ejemplo, un pendrive), el programa lo trae a su carpeta con sus adjuntos.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Reglas v16 firmadas: programa 0.7.2-prueba con descarga y huella
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reglas.xlsx
+++ b/reglas.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -491,7 +491,7 @@
         </is>
       </c>
       <c r="B1" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>46321</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="3">
@@ -512,7 +512,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>0.7.1-prueba</t>
+          <t>0.7.2-prueba</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.7.1-prueba/Instalar-GuiaRendicion-0.7.1-prueba.exe</t>
+          <t>https://github.com/georgeaguilera/guia-rendicion-reglas/releases/download/v0.7.2-prueba/Instalar-GuiaRendicion-0.7.2-prueba.exe</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>639C374DA247FA0E9BA73B2EBC0A40D4AC3F3AB3FC6E85BCFFE43D7FCC73D518</t>
+          <t>A0E80D9746B508A243145072302073092EE034C96B70C0AC2708D856141079DC</t>
         </is>
       </c>
     </row>
@@ -730,166 +730,178 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Cambios en la versión 15</t>
+          <t>Cambios en la versión 16</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>La novedad de la versión 14 ya no menciona la versión web, que se descartó el 26-10-2026: el programa es solo para Windows. Ninguna regla cambia.</t>
+          <t>Programa 0.7.2-prueba, con el ícono nuevo, y su instalador publicado como release en GitHub (filas Descarga y Huella). Ninguna regla cambia.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cambios en la versión 14</t>
+          <t>Cambios en la versión 15</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Textos de esta hoja: la firma al publicar (paso 8), de dónde salen las Fuentes (paso 18), el canal de prueba (paso 19) y la fila Contenido. Programa 0.7.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella), y una novedad para ese programa: adjuntos, montos y copias del proyecto.</t>
+          <t>La novedad de la versión 14 ya no menciona la versión web, que se descartó el 26-10-2026: el programa es solo para Windows. Ninguna regla cambia.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cambios en la versión 13</t>
+          <t>Cambios en la versión 14</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Hojas Retenciones (honorarios 2026 a 2028) y Fuentes (87 normas y documentos con su enlace oficial). Una novedad para el programa 0.7.0-prueba: presupuesto, revisión de documentos, carpeta para SISREC, informe IN17, avisos y Biblioteca.</t>
+          <t>Textos de esta hoja: la firma al publicar (paso 8), de dónde salen las Fuentes (paso 18), el canal de prueba (paso 19) y la fila Contenido. Programa 0.7.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella), y una novedad para ese programa: adjuntos, montos y copias del proyecto.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cambios en la versión 12</t>
+          <t>Cambios en la versión 13</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
+          <t>Hojas Retenciones (honorarios 2026 a 2028) y Fuentes (87 normas y documentos con su enlace oficial). Una novedad para el programa 0.7.0-prueba: presupuesto, revisión de documentos, carpeta para SISREC, informe IN17, avisos y Biblioteca.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cambios en la versión 11</t>
+          <t>Cambios en la versión 12</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
+          <t>Programa 0.6.1-prueba, con su instalador publicado como release en GitHub (filas Descarga y Huella). Prórroga: si el convenio no tiene fecha de vencimiento, los 30 días se cuentan desde el término de la ejecución (Plazos, Etapas, Situaciones y Glosario), y la contradicción queda en «Pendiente de validar». Una novedad para el programa 0.6.1-prueba: fecha de aceptación en SISREC, prórroga y garantía en el calendario.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cambios en la versión 10</t>
+          <t>Cambios en la versión 11</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
+          <t>Programa 0.6.0-prueba, con su instalador publicado como release en GitHub (fila Descarga) y la fila nueva Huella, que permite la actualización automática.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cambios en la versión 9</t>
+          <t>Cambios en la versión 10</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
+          <t>Hojas Situaciones («¿Qué hago si…?», con la Sección 3.01 de la Rex 3096 y la Rex 3097) y SISREC (7 trámites resumidos de los manuales del ejecutor de la Contraloría, con su enlace).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cambios en la versión 8</t>
+          <t>Cambios en la versión 9</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
+          <t>Programa 0.4.0-prueba: proyecto guardado, menú lateral, «Tu próximo paso» y seguimiento de documentos y verificadores. Una novedad que lo anuncia, solo para ese programa o uno posterior.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cambios en la versión 7</t>
+          <t>Cambios en la versión 8</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
+          <t>Columna DesdePrograma en Novedades: cada novedad se muestra solo en los programas que tienen lo que anuncia. La de «Así avanza tu proyecto» (versión 7) queda desde el programa 0.3.1-prueba.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cambios en la versión 6</t>
+          <t>Cambios en la versión 7</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
+          <t>Hoja Etapas: «Así avanza tu proyecto», las 7 etapas del convenio y el desvío para pedir cambios, con lo que haces tú, lo que hace el Ministerio y los plazos de cada norma (textos aprobados el 19-10-2026). VigenteDesde y VigenteHasta se comparan con la fecha de firma.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cambios en la versión 5</t>
+          <t>Cambios en la versión 6</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
+          <t>Hojas Feriados (2026 a 2028, desde las leyes de cada feriado), Topes (imprevistos y asignación del responsable de las bases 2027) y Glosario (16 términos).</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Cambios en la versión 4</t>
+          <t>Cambios en la versión 5</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
+          <t>Filas Programa y Descarga en esta hoja, para el aviso de versión nueva del programa.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Cambios en la versión 3</t>
+          <t>Cambios en la versión 4</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+          <t>Con los documentos de «Biblioteca Transferencias»: SISREC según la norma (excepción de 500 UTM con la Res. 30), rendiciones pendientes iguales en ambas normas, cambios dentro de un ítem según el convenio, gastos anteriores, fuerza mayor, tarjeta de crédito, documentos perdidos, copias de facturas, indemnizaciones voluntarias e inicio de actividades.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>Cambios en la versión 3</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Hoja Novedades: el programa avisa al responsable lo que cambió desde la última versión que leyó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t>Cambios en la versión 2</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Plazos corregidos con la matriz de plazos (gradualidad de la Res. 2/2026, renovación de la letra, segundo aviso). Respaldos contrastados con el Anexo A de la Rex 3391. SISREC para todos (Memo 02/566). Reglas del Fondo Audiovisual (Rex 3390). Subítem Viáticos y palabras clave de traslados. Bases 2027 de la tanda 1 en ReglasBases.</t>
         </is>

</xml_diff>